<commit_message>
Update legacy report data
</commit_message>
<xml_diff>
--- a/data/monthly/【2025年10月】月次数値.xlsx
+++ b/data/monthly/【2025年10月】月次数値.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="163">
   <si>
     <t>レポート開始日</t>
   </si>
@@ -275,6 +275,264 @@
   </si>
   <si>
     <t>銀座トレーニングラボ</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【Dining Bar Lien】...</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 📍町寿司いちもんめ｜福井市大手...</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌸【女性クリニック ラポール】🌸
+すべての世代の女性に、安心と寄り添いを。...</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【髙橋歯科】
+“噛み合わせ”から整える、お口とカラダのトータルケア🪥...</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 📍Wild Crepes - ワイルドクレープス
+安い！旨い！多い！🎉...</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍸【bar moon walk 三条木屋町店】🌙...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍶【駕町 とくさ】熊本・花畑町駅 徒歩5分...</t>
+  </si>
+  <si>
+    <t>炭焼　猿一</t>
+  </si>
+  <si>
+    <t>2026-01-15</t>
+  </si>
+  <si>
+    <t>島田屋　東苗穂店</t>
+  </si>
+  <si>
+    <t>居ZAKKU　CHENOWA</t>
+  </si>
+  <si>
+    <t>三千段の民宿　幸登里</t>
+  </si>
+  <si>
+    <t>てんぐ屋</t>
+  </si>
+  <si>
+    <t>炭火焼肉友丸</t>
+  </si>
+  <si>
+    <t>旬彩屋　笑味</t>
+  </si>
+  <si>
+    <t>有限会社　大嶋_うまか喰い処 祇園 大しま</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【海鮮と肉料理 ほっかい酒房】🍣🍢✨
+すすきの駅から徒歩3分🚶‍♂️...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【せがわ歯科クリニック】です🦷✨...</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【ORINAS】です🍽️✨...</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【CasualClub青】です🎤✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【Mix Bar Blo】です🍸✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【はんすう】です🍦✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【すし嘉まさ】🍣✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【すし嘉まさ】新しい仲間を募集しています！🍣✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【鮨一花】🍣✨
+豊水すすきの駅から徒歩1分🚶‍♂️🎶...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 新潟県長岡市に佇むカフェ『樹林館』🌳☕️...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 「新潟県長岡市に佇むカフェ『樹林館』🌳☕️...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍴肴家 信清🍷...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 家系ラーメン武将家　浅草店
+10月5日にオープンした『家系らーめん...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 「SEA DROP Roast...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍽️【特別な日のご褒美に】...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 和牛焼肉としお
+🥩和牛焼肉の新境地へ— 🥩...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【駅チカ×喫煙OK×最新機種】🎤✨...</t>
+  </si>
+  <si>
+    <t>archived</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍜日々“育てる”一杯、ここにあり🔥...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍷✨クオリティ高×価格安×lowkeyな接客✨🍴...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: ✨2024年9月20日 NEW OPEN✨
+Hairsalon...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【Meibuキッズ空手教室】
+＼2〜3歳のお子さまも大歓迎👶✨／...</t>
+  </si>
+  <si>
+    <t>2026-01-02</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 【Meibuキッズ空手教室】
+＼ドキドキ💓はじめてのスポーツ体験！／...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: インプラント治療なら「上志津中央歯科」🌟...</t>
+  </si>
+  <si>
+    <t>recently_completed</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 中洲にあるミュージックカラオケバー！Food持ち込み可🍴🎶...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🔥【香り豊かな炭火焼と多彩な日本酒が楽しめる！】🔥...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: んにちは！【Mont Blanc】です🍸✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟SUNRISEガールズバー｜豊田市山之手🌟...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍷 株式会社 TechVoice・FRETTA 🍸
+✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 📢 株式会社 TechVoice・FRETTA スタッフ募集中！ 🍸
+✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🏡☕canurip Cafe☕🏡
+茨木に佇む韓国風古民家カフェღ...</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍻 鉄板居酒屋こぐま 🔥
+🏡 アットホームな空間で、心もお腹も大満足！...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 至福のひとときを、すすきの 蟹一 で。
+✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍶 合同会社 大和・北海道の幸とお酒 たかふじ 🐟
+✨...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: ✨ 天ぷら むらやま｜吉祥寺 ✨
+ゆったりとした カウンター席...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 遠心太助 – 新発想の洗浄ツールで塗装コスト削減！ 🌍
+🔹...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍷 pikku onni 🍽️
+🐟 北海道の海の恵み ×...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🥩 焼肉処 縁結び｜鮮度抜群の極上焼肉 🥩...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🎤 カラオケサーカス 調布店 🎪✨
+東京・調布市の音楽オアシス！🌆🎶...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟大林歯科医院｜千葉県美浜区幕張西🌟...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟栄駅から徒歩2分の歯医者【日生歯科診療所】🌟...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟府中市の歯医者【たかすぎ歯科クリニック】🌟...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟かわらもと歯科｜大阪市・吹田市🌟...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🍻【リーズナブルにたくさん食べたいなら「居酒屋一（ichi）」】🍻...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: ✨【国分町に新しい刺激を！】✨
+「Extreme Bar...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌻季節の食材を使った心温まるお料理とお酒🌻...</t>
+  </si>
+  <si>
+    <t>2026-09-29</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌟【焼鳥の真髄、ここにあり】🌟
+「焼鳥酒場...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🌙【川越の夜をおしゃれに楽しむならここ！】🌙
+「AMUSEMENT Bar...</t>
+  </si>
+  <si>
+    <t>Instagram投稿: 🐾✨ Heart Dog ✨🐶
+ドッグカフェ 庵（いおり） OPEN！...</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
   </si>
 </sst>
 </file>
@@ -624,7 +882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:Y99"/>
   <sheetFormatPr defaultColWidth="20" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">
@@ -2852,6 +3110,4682 @@
       </c>
       <c r="Y32">
         <v>42.267175999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" t="s">
+        <v>38</v>
+      </c>
+      <c r="E33" t="s">
+        <v>29</v>
+      </c>
+      <c r="F33">
+        <v>136</v>
+      </c>
+      <c r="G33" t="s">
+        <v>42</v>
+      </c>
+      <c r="H33">
+        <v>4541</v>
+      </c>
+      <c r="I33">
+        <v>1.5223519999999999</v>
+      </c>
+      <c r="J33">
+        <v>36.169117649999997</v>
+      </c>
+      <c r="K33">
+        <v>160</v>
+      </c>
+      <c r="L33" t="s">
+        <v>30</v>
+      </c>
+      <c r="M33">
+        <v>4919</v>
+      </c>
+      <c r="N33" t="s">
+        <v>86</v>
+      </c>
+      <c r="O33">
+        <v>6913</v>
+      </c>
+      <c r="P33">
+        <v>711.55793400000005</v>
+      </c>
+      <c r="Q33">
+        <v>136</v>
+      </c>
+      <c r="S33">
+        <v>36.169117999999997</v>
+      </c>
+      <c r="T33">
+        <v>1.9673080000000001</v>
+      </c>
+      <c r="U33">
+        <v>181</v>
+      </c>
+      <c r="V33">
+        <v>2.618255</v>
+      </c>
+      <c r="W33">
+        <v>27.176796</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D34" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" t="s">
+        <v>29</v>
+      </c>
+      <c r="F34">
+        <v>24</v>
+      </c>
+      <c r="G34" t="s">
+        <v>42</v>
+      </c>
+      <c r="H34">
+        <v>479</v>
+      </c>
+      <c r="I34">
+        <v>1.139875</v>
+      </c>
+      <c r="J34">
+        <v>43.791666669999998</v>
+      </c>
+      <c r="K34">
+        <v>160</v>
+      </c>
+      <c r="L34" t="s">
+        <v>30</v>
+      </c>
+      <c r="M34">
+        <v>1051</v>
+      </c>
+      <c r="N34" t="s">
+        <v>88</v>
+      </c>
+      <c r="O34">
+        <v>546</v>
+      </c>
+      <c r="P34">
+        <v>1924.9084250000001</v>
+      </c>
+      <c r="Q34">
+        <v>24</v>
+      </c>
+      <c r="S34">
+        <v>43.791666999999997</v>
+      </c>
+      <c r="T34">
+        <v>4.3956039999999996</v>
+      </c>
+      <c r="U34">
+        <v>25</v>
+      </c>
+      <c r="V34">
+        <v>4.5787550000000001</v>
+      </c>
+      <c r="W34">
+        <v>42.04</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35">
+        <v>97</v>
+      </c>
+      <c r="G35" t="s">
+        <v>42</v>
+      </c>
+      <c r="H35">
+        <v>2796</v>
+      </c>
+      <c r="I35">
+        <v>1.6863379999999999</v>
+      </c>
+      <c r="J35">
+        <v>50.855670099999998</v>
+      </c>
+      <c r="K35">
+        <v>160</v>
+      </c>
+      <c r="L35" t="s">
+        <v>30</v>
+      </c>
+      <c r="M35">
+        <v>4933</v>
+      </c>
+      <c r="N35" t="s">
+        <v>90</v>
+      </c>
+      <c r="O35">
+        <v>4715</v>
+      </c>
+      <c r="P35">
+        <v>1046.2354190000001</v>
+      </c>
+      <c r="Q35">
+        <v>97</v>
+      </c>
+      <c r="S35">
+        <v>50.855670000000003</v>
+      </c>
+      <c r="T35">
+        <v>2.057264</v>
+      </c>
+      <c r="U35">
+        <v>120</v>
+      </c>
+      <c r="V35">
+        <v>2.5450689999999998</v>
+      </c>
+      <c r="W35">
+        <v>41.108333000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" t="s">
+        <v>91</v>
+      </c>
+      <c r="D36" t="s">
+        <v>28</v>
+      </c>
+      <c r="E36" t="s">
+        <v>29</v>
+      </c>
+      <c r="H36">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>160</v>
+      </c>
+      <c r="L36" t="s">
+        <v>30</v>
+      </c>
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36" t="s">
+        <v>92</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <v>0</v>
+      </c>
+      <c r="U36">
+        <v>0</v>
+      </c>
+      <c r="V36">
+        <v>0</v>
+      </c>
+      <c r="W36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37">
+        <v>215</v>
+      </c>
+      <c r="G37" t="s">
+        <v>42</v>
+      </c>
+      <c r="H37">
+        <v>4496</v>
+      </c>
+      <c r="I37">
+        <v>1.4762010000000001</v>
+      </c>
+      <c r="J37">
+        <v>22.916279070000002</v>
+      </c>
+      <c r="K37">
+        <v>160</v>
+      </c>
+      <c r="L37" t="s">
+        <v>30</v>
+      </c>
+      <c r="M37">
+        <v>4927</v>
+      </c>
+      <c r="N37" t="s">
+        <v>94</v>
+      </c>
+      <c r="O37">
+        <v>6637</v>
+      </c>
+      <c r="P37">
+        <v>742.35347300000001</v>
+      </c>
+      <c r="Q37">
+        <v>215</v>
+      </c>
+      <c r="S37">
+        <v>22.916278999999999</v>
+      </c>
+      <c r="T37">
+        <v>3.2394150000000002</v>
+      </c>
+      <c r="U37">
+        <v>261</v>
+      </c>
+      <c r="V37">
+        <v>3.9325000000000001</v>
+      </c>
+      <c r="W37">
+        <v>18.877395</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" t="s">
+        <v>95</v>
+      </c>
+      <c r="D38" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38">
+        <v>68</v>
+      </c>
+      <c r="G38" t="s">
+        <v>42</v>
+      </c>
+      <c r="H38">
+        <v>1643</v>
+      </c>
+      <c r="I38">
+        <v>1.277541</v>
+      </c>
+      <c r="J38">
+        <v>72.352941180000002</v>
+      </c>
+      <c r="K38">
+        <v>160</v>
+      </c>
+      <c r="L38" t="s">
+        <v>30</v>
+      </c>
+      <c r="M38">
+        <v>4920</v>
+      </c>
+      <c r="N38" t="s">
+        <v>94</v>
+      </c>
+      <c r="O38">
+        <v>2099</v>
+      </c>
+      <c r="P38">
+        <v>2343.9733209999999</v>
+      </c>
+      <c r="Q38">
+        <v>68</v>
+      </c>
+      <c r="S38">
+        <v>72.352941000000001</v>
+      </c>
+      <c r="T38">
+        <v>3.2396379999999998</v>
+      </c>
+      <c r="U38">
+        <v>75</v>
+      </c>
+      <c r="V38">
+        <v>3.5731299999999999</v>
+      </c>
+      <c r="W38">
+        <v>65.599999999999994</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" t="s">
+        <v>29</v>
+      </c>
+      <c r="F39">
+        <v>282</v>
+      </c>
+      <c r="G39" t="s">
+        <v>42</v>
+      </c>
+      <c r="H39">
+        <v>3612</v>
+      </c>
+      <c r="I39">
+        <v>1.6528240000000001</v>
+      </c>
+      <c r="J39">
+        <v>17.42553191</v>
+      </c>
+      <c r="K39">
+        <v>160</v>
+      </c>
+      <c r="L39" t="s">
+        <v>30</v>
+      </c>
+      <c r="M39">
+        <v>4914</v>
+      </c>
+      <c r="N39" t="s">
+        <v>94</v>
+      </c>
+      <c r="O39">
+        <v>5970</v>
+      </c>
+      <c r="P39">
+        <v>823.11557800000003</v>
+      </c>
+      <c r="Q39">
+        <v>282</v>
+      </c>
+      <c r="S39">
+        <v>17.425532</v>
+      </c>
+      <c r="T39">
+        <v>4.7236180000000001</v>
+      </c>
+      <c r="U39">
+        <v>320</v>
+      </c>
+      <c r="V39">
+        <v>5.3601340000000004</v>
+      </c>
+      <c r="W39">
+        <v>15.356249999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" t="s">
+        <v>97</v>
+      </c>
+      <c r="D40" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" t="s">
+        <v>29</v>
+      </c>
+      <c r="F40">
+        <v>330</v>
+      </c>
+      <c r="G40" t="s">
+        <v>42</v>
+      </c>
+      <c r="H40">
+        <v>5449</v>
+      </c>
+      <c r="I40">
+        <v>1.553129</v>
+      </c>
+      <c r="J40">
+        <v>16.38181818</v>
+      </c>
+      <c r="K40" t="s">
+        <v>34</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
+        <v>5406</v>
+      </c>
+      <c r="N40" t="s">
+        <v>98</v>
+      </c>
+      <c r="O40">
+        <v>8463</v>
+      </c>
+      <c r="P40">
+        <v>638.780574</v>
+      </c>
+      <c r="Q40">
+        <v>330</v>
+      </c>
+      <c r="S40">
+        <v>16.381817999999999</v>
+      </c>
+      <c r="T40">
+        <v>3.8993259999999998</v>
+      </c>
+      <c r="U40">
+        <v>368</v>
+      </c>
+      <c r="V40">
+        <v>4.3483400000000003</v>
+      </c>
+      <c r="W40">
+        <v>14.690217000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
+        <v>26</v>
+      </c>
+      <c r="C41" t="s">
+        <v>99</v>
+      </c>
+      <c r="D41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" t="s">
+        <v>29</v>
+      </c>
+      <c r="F41">
+        <v>326</v>
+      </c>
+      <c r="G41" t="s">
+        <v>42</v>
+      </c>
+      <c r="H41">
+        <v>6717</v>
+      </c>
+      <c r="I41">
+        <v>1.5433969999999999</v>
+      </c>
+      <c r="J41">
+        <v>16.352760740000001</v>
+      </c>
+      <c r="K41" t="s">
+        <v>34</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>5331</v>
+      </c>
+      <c r="N41" t="s">
+        <v>98</v>
+      </c>
+      <c r="O41">
+        <v>10367</v>
+      </c>
+      <c r="P41">
+        <v>514.22783800000002</v>
+      </c>
+      <c r="Q41">
+        <v>326</v>
+      </c>
+      <c r="S41">
+        <v>16.352761000000001</v>
+      </c>
+      <c r="T41">
+        <v>3.144593</v>
+      </c>
+      <c r="U41">
+        <v>359</v>
+      </c>
+      <c r="V41">
+        <v>3.4629110000000001</v>
+      </c>
+      <c r="W41">
+        <v>14.849582</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>25</v>
+      </c>
+      <c r="B42" t="s">
+        <v>26</v>
+      </c>
+      <c r="C42" t="s">
+        <v>100</v>
+      </c>
+      <c r="D42" t="s">
+        <v>38</v>
+      </c>
+      <c r="E42" t="s">
+        <v>29</v>
+      </c>
+      <c r="F42">
+        <v>160</v>
+      </c>
+      <c r="G42" t="s">
+        <v>42</v>
+      </c>
+      <c r="H42">
+        <v>4039</v>
+      </c>
+      <c r="I42">
+        <v>1.697697</v>
+      </c>
+      <c r="J42">
+        <v>37.46875</v>
+      </c>
+      <c r="K42" t="s">
+        <v>34</v>
+      </c>
+      <c r="L42">
+        <v>0</v>
+      </c>
+      <c r="M42">
+        <v>5995</v>
+      </c>
+      <c r="N42" t="s">
+        <v>35</v>
+      </c>
+      <c r="O42">
+        <v>6857</v>
+      </c>
+      <c r="P42">
+        <v>874.28904799999998</v>
+      </c>
+      <c r="Q42">
+        <v>160</v>
+      </c>
+      <c r="S42">
+        <v>37.46875</v>
+      </c>
+      <c r="T42">
+        <v>2.3333819999999998</v>
+      </c>
+      <c r="U42">
+        <v>197</v>
+      </c>
+      <c r="V42">
+        <v>2.8729770000000001</v>
+      </c>
+      <c r="W42">
+        <v>30.431471999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" t="s">
+        <v>101</v>
+      </c>
+      <c r="D43" t="s">
+        <v>38</v>
+      </c>
+      <c r="E43" t="s">
+        <v>29</v>
+      </c>
+      <c r="F43">
+        <v>184</v>
+      </c>
+      <c r="G43" t="s">
+        <v>42</v>
+      </c>
+      <c r="H43">
+        <v>3407</v>
+      </c>
+      <c r="I43">
+        <v>1.4285300000000001</v>
+      </c>
+      <c r="J43">
+        <v>30.25</v>
+      </c>
+      <c r="K43" t="s">
+        <v>34</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43">
+        <v>5566</v>
+      </c>
+      <c r="N43" t="s">
+        <v>98</v>
+      </c>
+      <c r="O43">
+        <v>4867</v>
+      </c>
+      <c r="P43">
+        <v>1143.6203</v>
+      </c>
+      <c r="Q43">
+        <v>184</v>
+      </c>
+      <c r="S43">
+        <v>30.25</v>
+      </c>
+      <c r="T43">
+        <v>3.7805629999999999</v>
+      </c>
+      <c r="U43">
+        <v>202</v>
+      </c>
+      <c r="V43">
+        <v>4.1504009999999996</v>
+      </c>
+      <c r="W43">
+        <v>27.554455000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" t="s">
+        <v>102</v>
+      </c>
+      <c r="D44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E44" t="s">
+        <v>29</v>
+      </c>
+      <c r="F44">
+        <v>443</v>
+      </c>
+      <c r="G44" t="s">
+        <v>42</v>
+      </c>
+      <c r="H44">
+        <v>5382</v>
+      </c>
+      <c r="I44">
+        <v>1.471014</v>
+      </c>
+      <c r="J44">
+        <v>12.957110610000001</v>
+      </c>
+      <c r="K44" t="s">
+        <v>34</v>
+      </c>
+      <c r="L44">
+        <v>0</v>
+      </c>
+      <c r="M44">
+        <v>5740</v>
+      </c>
+      <c r="N44" t="s">
+        <v>35</v>
+      </c>
+      <c r="O44">
+        <v>7917</v>
+      </c>
+      <c r="P44">
+        <v>725.02210400000001</v>
+      </c>
+      <c r="Q44">
+        <v>443</v>
+      </c>
+      <c r="S44">
+        <v>12.957110999999999</v>
+      </c>
+      <c r="T44">
+        <v>5.5955539999999999</v>
+      </c>
+      <c r="U44">
+        <v>472</v>
+      </c>
+      <c r="V44">
+        <v>5.9618539999999998</v>
+      </c>
+      <c r="W44">
+        <v>12.161016999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" t="s">
+        <v>26</v>
+      </c>
+      <c r="C45" t="s">
+        <v>103</v>
+      </c>
+      <c r="D45" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" t="s">
+        <v>29</v>
+      </c>
+      <c r="F45">
+        <v>180</v>
+      </c>
+      <c r="G45" t="s">
+        <v>42</v>
+      </c>
+      <c r="H45">
+        <v>5604</v>
+      </c>
+      <c r="I45">
+        <v>1.544611</v>
+      </c>
+      <c r="J45">
+        <v>32.022222220000003</v>
+      </c>
+      <c r="K45" t="s">
+        <v>34</v>
+      </c>
+      <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
+        <v>5764</v>
+      </c>
+      <c r="N45" t="s">
+        <v>35</v>
+      </c>
+      <c r="O45">
+        <v>8656</v>
+      </c>
+      <c r="P45">
+        <v>665.89648799999998</v>
+      </c>
+      <c r="Q45">
+        <v>180</v>
+      </c>
+      <c r="S45">
+        <v>32.022221999999999</v>
+      </c>
+      <c r="T45">
+        <v>2.0794820000000001</v>
+      </c>
+      <c r="U45">
+        <v>223</v>
+      </c>
+      <c r="V45">
+        <v>2.5762480000000001</v>
+      </c>
+      <c r="W45">
+        <v>25.847534</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>25</v>
+      </c>
+      <c r="B46" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" t="s">
+        <v>29</v>
+      </c>
+      <c r="F46">
+        <v>194</v>
+      </c>
+      <c r="G46" t="s">
+        <v>42</v>
+      </c>
+      <c r="H46">
+        <v>3666</v>
+      </c>
+      <c r="I46">
+        <v>1.7635019999999999</v>
+      </c>
+      <c r="J46">
+        <v>31.494845359999999</v>
+      </c>
+      <c r="K46" t="s">
+        <v>34</v>
+      </c>
+      <c r="L46">
+        <v>0</v>
+      </c>
+      <c r="M46">
+        <v>6110</v>
+      </c>
+      <c r="N46" t="s">
+        <v>35</v>
+      </c>
+      <c r="O46">
+        <v>6465</v>
+      </c>
+      <c r="P46">
+        <v>945.08893999999998</v>
+      </c>
+      <c r="Q46">
+        <v>194</v>
+      </c>
+      <c r="S46">
+        <v>31.494845000000002</v>
+      </c>
+      <c r="T46">
+        <v>3.0007730000000001</v>
+      </c>
+      <c r="U46">
+        <v>235</v>
+      </c>
+      <c r="V46">
+        <v>3.634957</v>
+      </c>
+      <c r="W46">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" t="s">
+        <v>26</v>
+      </c>
+      <c r="C47" t="s">
+        <v>105</v>
+      </c>
+      <c r="D47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E47" t="s">
+        <v>29</v>
+      </c>
+      <c r="F47">
+        <v>299</v>
+      </c>
+      <c r="G47" t="s">
+        <v>42</v>
+      </c>
+      <c r="H47">
+        <v>4694</v>
+      </c>
+      <c r="I47">
+        <v>1.521091</v>
+      </c>
+      <c r="J47">
+        <v>19.779264210000001</v>
+      </c>
+      <c r="K47" t="s">
+        <v>34</v>
+      </c>
+      <c r="L47">
+        <v>0</v>
+      </c>
+      <c r="M47">
+        <v>5914</v>
+      </c>
+      <c r="N47" t="s">
+        <v>80</v>
+      </c>
+      <c r="O47">
+        <v>7140</v>
+      </c>
+      <c r="P47">
+        <v>828.29131700000005</v>
+      </c>
+      <c r="Q47">
+        <v>299</v>
+      </c>
+      <c r="S47">
+        <v>19.779264000000001</v>
+      </c>
+      <c r="T47">
+        <v>4.1876749999999996</v>
+      </c>
+      <c r="U47">
+        <v>334</v>
+      </c>
+      <c r="V47">
+        <v>4.6778709999999997</v>
+      </c>
+      <c r="W47">
+        <v>17.706586999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>25</v>
+      </c>
+      <c r="B48" t="s">
+        <v>26</v>
+      </c>
+      <c r="C48" t="s">
+        <v>106</v>
+      </c>
+      <c r="D48" t="s">
+        <v>38</v>
+      </c>
+      <c r="E48" t="s">
+        <v>29</v>
+      </c>
+      <c r="F48">
+        <v>292</v>
+      </c>
+      <c r="G48" t="s">
+        <v>42</v>
+      </c>
+      <c r="H48">
+        <v>4211</v>
+      </c>
+      <c r="I48">
+        <v>1.4511989999999999</v>
+      </c>
+      <c r="J48">
+        <v>16.770547950000001</v>
+      </c>
+      <c r="K48">
+        <v>160</v>
+      </c>
+      <c r="L48" t="s">
+        <v>30</v>
+      </c>
+      <c r="M48">
+        <v>4897</v>
+      </c>
+      <c r="N48" t="s">
+        <v>70</v>
+      </c>
+      <c r="O48">
+        <v>6111</v>
+      </c>
+      <c r="P48">
+        <v>801.34184300000004</v>
+      </c>
+      <c r="Q48">
+        <v>292</v>
+      </c>
+      <c r="S48">
+        <v>16.770548000000002</v>
+      </c>
+      <c r="T48">
+        <v>4.7782689999999999</v>
+      </c>
+      <c r="U48">
+        <v>318</v>
+      </c>
+      <c r="V48">
+        <v>5.2037310000000003</v>
+      </c>
+      <c r="W48">
+        <v>15.399371</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49" t="s">
+        <v>107</v>
+      </c>
+      <c r="D49" t="s">
+        <v>38</v>
+      </c>
+      <c r="E49" t="s">
+        <v>29</v>
+      </c>
+      <c r="F49">
+        <v>94</v>
+      </c>
+      <c r="G49" t="s">
+        <v>42</v>
+      </c>
+      <c r="H49">
+        <v>4267</v>
+      </c>
+      <c r="I49">
+        <v>1.3248180000000001</v>
+      </c>
+      <c r="J49">
+        <v>52.595744680000003</v>
+      </c>
+      <c r="K49">
+        <v>160</v>
+      </c>
+      <c r="L49" t="s">
+        <v>30</v>
+      </c>
+      <c r="M49">
+        <v>4944</v>
+      </c>
+      <c r="N49" t="s">
+        <v>108</v>
+      </c>
+      <c r="O49">
+        <v>5653</v>
+      </c>
+      <c r="P49">
+        <v>874.57986900000003</v>
+      </c>
+      <c r="Q49">
+        <v>94</v>
+      </c>
+      <c r="S49">
+        <v>52.595745000000001</v>
+      </c>
+      <c r="T49">
+        <v>1.6628339999999999</v>
+      </c>
+      <c r="U49">
+        <v>113</v>
+      </c>
+      <c r="V49">
+        <v>1.998939</v>
+      </c>
+      <c r="W49">
+        <v>43.752212</v>
+      </c>
+      <c r="X49">
+        <v>83</v>
+      </c>
+      <c r="Y49">
+        <v>59.566265000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" t="s">
+        <v>26</v>
+      </c>
+      <c r="C50" t="s">
+        <v>109</v>
+      </c>
+      <c r="D50" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" t="s">
+        <v>29</v>
+      </c>
+      <c r="F50">
+        <v>254</v>
+      </c>
+      <c r="G50" t="s">
+        <v>42</v>
+      </c>
+      <c r="H50">
+        <v>3543</v>
+      </c>
+      <c r="I50">
+        <v>1.622072</v>
+      </c>
+      <c r="J50">
+        <v>19.33464567</v>
+      </c>
+      <c r="K50">
+        <v>160</v>
+      </c>
+      <c r="L50" t="s">
+        <v>30</v>
+      </c>
+      <c r="M50">
+        <v>4911</v>
+      </c>
+      <c r="N50" t="s">
+        <v>110</v>
+      </c>
+      <c r="O50">
+        <v>5747</v>
+      </c>
+      <c r="P50">
+        <v>854.53279999999995</v>
+      </c>
+      <c r="Q50">
+        <v>254</v>
+      </c>
+      <c r="S50">
+        <v>19.334645999999999</v>
+      </c>
+      <c r="T50">
+        <v>4.4196970000000002</v>
+      </c>
+      <c r="U50">
+        <v>270</v>
+      </c>
+      <c r="V50">
+        <v>4.6981029999999997</v>
+      </c>
+      <c r="W50">
+        <v>18.188889</v>
+      </c>
+      <c r="X50">
+        <v>226</v>
+      </c>
+      <c r="Y50">
+        <v>21.730089</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D51" t="s">
+        <v>38</v>
+      </c>
+      <c r="E51" t="s">
+        <v>29</v>
+      </c>
+      <c r="F51">
+        <v>189</v>
+      </c>
+      <c r="G51" t="s">
+        <v>42</v>
+      </c>
+      <c r="H51">
+        <v>4704</v>
+      </c>
+      <c r="I51">
+        <v>1.517857</v>
+      </c>
+      <c r="J51">
+        <v>26.11111111</v>
+      </c>
+      <c r="K51">
+        <v>160</v>
+      </c>
+      <c r="L51" t="s">
+        <v>30</v>
+      </c>
+      <c r="M51">
+        <v>4935</v>
+      </c>
+      <c r="N51" t="s">
+        <v>110</v>
+      </c>
+      <c r="O51">
+        <v>7140</v>
+      </c>
+      <c r="P51">
+        <v>691.17647099999999</v>
+      </c>
+      <c r="Q51">
+        <v>189</v>
+      </c>
+      <c r="S51">
+        <v>26.111111000000001</v>
+      </c>
+      <c r="T51">
+        <v>2.6470590000000001</v>
+      </c>
+      <c r="U51">
+        <v>224</v>
+      </c>
+      <c r="V51">
+        <v>3.1372550000000001</v>
+      </c>
+      <c r="W51">
+        <v>22.03125</v>
+      </c>
+      <c r="X51">
+        <v>168</v>
+      </c>
+      <c r="Y51">
+        <v>29.375</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>25</v>
+      </c>
+      <c r="B52" t="s">
+        <v>26</v>
+      </c>
+      <c r="C52" t="s">
+        <v>112</v>
+      </c>
+      <c r="D52" t="s">
+        <v>38</v>
+      </c>
+      <c r="E52" t="s">
+        <v>29</v>
+      </c>
+      <c r="F52">
+        <v>231</v>
+      </c>
+      <c r="G52" t="s">
+        <v>42</v>
+      </c>
+      <c r="H52">
+        <v>3840</v>
+      </c>
+      <c r="I52">
+        <v>1.79375</v>
+      </c>
+      <c r="J52">
+        <v>21.372294369999999</v>
+      </c>
+      <c r="K52">
+        <v>160</v>
+      </c>
+      <c r="L52" t="s">
+        <v>30</v>
+      </c>
+      <c r="M52">
+        <v>4937</v>
+      </c>
+      <c r="N52" t="s">
+        <v>110</v>
+      </c>
+      <c r="O52">
+        <v>6888</v>
+      </c>
+      <c r="P52">
+        <v>716.75377500000002</v>
+      </c>
+      <c r="Q52">
+        <v>231</v>
+      </c>
+      <c r="S52">
+        <v>21.372294</v>
+      </c>
+      <c r="T52">
+        <v>3.3536589999999999</v>
+      </c>
+      <c r="U52">
+        <v>311</v>
+      </c>
+      <c r="V52">
+        <v>4.5150990000000002</v>
+      </c>
+      <c r="W52">
+        <v>15.874598000000001</v>
+      </c>
+      <c r="X52">
+        <v>64</v>
+      </c>
+      <c r="Y52">
+        <v>77.140625</v>
+      </c>
+    </row>
+    <row r="53" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>25</v>
+      </c>
+      <c r="B53" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" t="s">
+        <v>113</v>
+      </c>
+      <c r="D53" t="s">
+        <v>38</v>
+      </c>
+      <c r="E53" t="s">
+        <v>29</v>
+      </c>
+      <c r="F53">
+        <v>105</v>
+      </c>
+      <c r="G53" t="s">
+        <v>42</v>
+      </c>
+      <c r="H53">
+        <v>3319</v>
+      </c>
+      <c r="I53">
+        <v>1.587526</v>
+      </c>
+      <c r="J53">
+        <v>46.79047619</v>
+      </c>
+      <c r="K53">
+        <v>160</v>
+      </c>
+      <c r="L53" t="s">
+        <v>30</v>
+      </c>
+      <c r="M53">
+        <v>4913</v>
+      </c>
+      <c r="N53" t="s">
+        <v>110</v>
+      </c>
+      <c r="O53">
+        <v>5269</v>
+      </c>
+      <c r="P53">
+        <v>932.43499699999995</v>
+      </c>
+      <c r="Q53">
+        <v>105</v>
+      </c>
+      <c r="S53">
+        <v>46.790475999999998</v>
+      </c>
+      <c r="T53">
+        <v>1.992788</v>
+      </c>
+      <c r="U53">
+        <v>146</v>
+      </c>
+      <c r="V53">
+        <v>2.7709239999999999</v>
+      </c>
+      <c r="W53">
+        <v>33.650685000000003</v>
+      </c>
+      <c r="X53">
+        <v>42</v>
+      </c>
+      <c r="Y53">
+        <v>116.97619</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>25</v>
+      </c>
+      <c r="B54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C54" t="s">
+        <v>114</v>
+      </c>
+      <c r="D54" t="s">
+        <v>28</v>
+      </c>
+      <c r="E54" t="s">
+        <v>29</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="K54">
+        <v>160</v>
+      </c>
+      <c r="L54" t="s">
+        <v>30</v>
+      </c>
+      <c r="M54">
+        <v>0</v>
+      </c>
+      <c r="N54" t="s">
+        <v>110</v>
+      </c>
+      <c r="O54">
+        <v>0</v>
+      </c>
+      <c r="P54">
+        <v>0</v>
+      </c>
+      <c r="U54">
+        <v>0</v>
+      </c>
+      <c r="V54">
+        <v>0</v>
+      </c>
+      <c r="W54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>25</v>
+      </c>
+      <c r="B55" t="s">
+        <v>26</v>
+      </c>
+      <c r="C55" t="s">
+        <v>115</v>
+      </c>
+      <c r="D55" t="s">
+        <v>28</v>
+      </c>
+      <c r="E55" t="s">
+        <v>29</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="K55">
+        <v>160</v>
+      </c>
+      <c r="L55" t="s">
+        <v>30</v>
+      </c>
+      <c r="M55">
+        <v>0</v>
+      </c>
+      <c r="N55" t="s">
+        <v>110</v>
+      </c>
+      <c r="O55">
+        <v>0</v>
+      </c>
+      <c r="P55">
+        <v>0</v>
+      </c>
+      <c r="U55">
+        <v>0</v>
+      </c>
+      <c r="V55">
+        <v>0</v>
+      </c>
+      <c r="W55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>25</v>
+      </c>
+      <c r="B56" t="s">
+        <v>26</v>
+      </c>
+      <c r="C56" t="s">
+        <v>116</v>
+      </c>
+      <c r="D56" t="s">
+        <v>28</v>
+      </c>
+      <c r="E56" t="s">
+        <v>29</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="K56">
+        <v>320</v>
+      </c>
+      <c r="L56" t="s">
+        <v>30</v>
+      </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+      <c r="N56" t="s">
+        <v>110</v>
+      </c>
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56">
+        <v>0</v>
+      </c>
+      <c r="U56">
+        <v>0</v>
+      </c>
+      <c r="V56">
+        <v>0</v>
+      </c>
+      <c r="W56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>25</v>
+      </c>
+      <c r="B57" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" t="s">
+        <v>117</v>
+      </c>
+      <c r="D57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E57" t="s">
+        <v>29</v>
+      </c>
+      <c r="F57">
+        <v>374</v>
+      </c>
+      <c r="G57" t="s">
+        <v>42</v>
+      </c>
+      <c r="H57">
+        <v>6735</v>
+      </c>
+      <c r="I57">
+        <v>1.4152929999999999</v>
+      </c>
+      <c r="J57">
+        <v>13.21122995</v>
+      </c>
+      <c r="K57">
+        <v>160</v>
+      </c>
+      <c r="L57" t="s">
+        <v>30</v>
+      </c>
+      <c r="M57">
+        <v>4941</v>
+      </c>
+      <c r="N57" t="s">
+        <v>110</v>
+      </c>
+      <c r="O57">
+        <v>9532</v>
+      </c>
+      <c r="P57">
+        <v>518.35921099999996</v>
+      </c>
+      <c r="Q57">
+        <v>374</v>
+      </c>
+      <c r="S57">
+        <v>13.21123</v>
+      </c>
+      <c r="T57">
+        <v>3.9236260000000001</v>
+      </c>
+      <c r="U57">
+        <v>438</v>
+      </c>
+      <c r="V57">
+        <v>4.5950480000000002</v>
+      </c>
+      <c r="W57">
+        <v>11.280822000000001</v>
+      </c>
+      <c r="X57">
+        <v>328</v>
+      </c>
+      <c r="Y57">
+        <v>15.064024</v>
+      </c>
+    </row>
+    <row r="58" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>25</v>
+      </c>
+      <c r="B58" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" t="s">
+        <v>118</v>
+      </c>
+      <c r="D58" t="s">
+        <v>38</v>
+      </c>
+      <c r="E58" t="s">
+        <v>29</v>
+      </c>
+      <c r="F58">
+        <v>337</v>
+      </c>
+      <c r="G58" t="s">
+        <v>42</v>
+      </c>
+      <c r="H58">
+        <v>7069</v>
+      </c>
+      <c r="I58">
+        <v>1.3290420000000001</v>
+      </c>
+      <c r="J58">
+        <v>14.602373890000001</v>
+      </c>
+      <c r="K58">
+        <v>160</v>
+      </c>
+      <c r="L58" t="s">
+        <v>30</v>
+      </c>
+      <c r="M58">
+        <v>4921</v>
+      </c>
+      <c r="N58" t="s">
+        <v>110</v>
+      </c>
+      <c r="O58">
+        <v>9395</v>
+      </c>
+      <c r="P58">
+        <v>523.78925000000004</v>
+      </c>
+      <c r="Q58">
+        <v>337</v>
+      </c>
+      <c r="S58">
+        <v>14.602373999999999</v>
+      </c>
+      <c r="T58">
+        <v>3.5870139999999999</v>
+      </c>
+      <c r="U58">
+        <v>481</v>
+      </c>
+      <c r="V58">
+        <v>5.119745</v>
+      </c>
+      <c r="W58">
+        <v>10.230769</v>
+      </c>
+      <c r="X58">
+        <v>314</v>
+      </c>
+      <c r="Y58">
+        <v>15.671975</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>25</v>
+      </c>
+      <c r="B59" t="s">
+        <v>26</v>
+      </c>
+      <c r="C59" t="s">
+        <v>119</v>
+      </c>
+      <c r="D59" t="s">
+        <v>38</v>
+      </c>
+      <c r="E59" t="s">
+        <v>29</v>
+      </c>
+      <c r="F59">
+        <v>64</v>
+      </c>
+      <c r="G59" t="s">
+        <v>42</v>
+      </c>
+      <c r="H59">
+        <v>2780</v>
+      </c>
+      <c r="I59">
+        <v>1.871583</v>
+      </c>
+      <c r="J59">
+        <v>76.484375</v>
+      </c>
+      <c r="K59">
+        <v>160</v>
+      </c>
+      <c r="L59" t="s">
+        <v>30</v>
+      </c>
+      <c r="M59">
+        <v>4895</v>
+      </c>
+      <c r="N59" t="s">
+        <v>110</v>
+      </c>
+      <c r="O59">
+        <v>5203</v>
+      </c>
+      <c r="P59">
+        <v>940.80338300000005</v>
+      </c>
+      <c r="Q59">
+        <v>64</v>
+      </c>
+      <c r="S59">
+        <v>76.484375</v>
+      </c>
+      <c r="T59">
+        <v>1.2300599999999999</v>
+      </c>
+      <c r="U59">
+        <v>71</v>
+      </c>
+      <c r="V59">
+        <v>1.3645970000000001</v>
+      </c>
+      <c r="W59">
+        <v>68.943662000000003</v>
+      </c>
+      <c r="X59">
+        <v>49</v>
+      </c>
+      <c r="Y59">
+        <v>99.897959</v>
+      </c>
+    </row>
+    <row r="60" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>25</v>
+      </c>
+      <c r="B60" t="s">
+        <v>26</v>
+      </c>
+      <c r="C60" t="s">
+        <v>120</v>
+      </c>
+      <c r="D60" t="s">
+        <v>38</v>
+      </c>
+      <c r="E60" t="s">
+        <v>29</v>
+      </c>
+      <c r="F60">
+        <v>793</v>
+      </c>
+      <c r="G60" t="s">
+        <v>42</v>
+      </c>
+      <c r="H60">
+        <v>10303</v>
+      </c>
+      <c r="I60">
+        <v>1.3513539999999999</v>
+      </c>
+      <c r="J60">
+        <v>6.2320302600000002</v>
+      </c>
+      <c r="K60">
+        <v>160</v>
+      </c>
+      <c r="L60" t="s">
+        <v>30</v>
+      </c>
+      <c r="M60">
+        <v>4942</v>
+      </c>
+      <c r="N60" t="s">
+        <v>110</v>
+      </c>
+      <c r="O60">
+        <v>13923</v>
+      </c>
+      <c r="P60">
+        <v>354.95223700000003</v>
+      </c>
+      <c r="Q60">
+        <v>793</v>
+      </c>
+      <c r="S60">
+        <v>6.23203</v>
+      </c>
+      <c r="T60">
+        <v>5.6956119999999997</v>
+      </c>
+      <c r="U60">
+        <v>922</v>
+      </c>
+      <c r="V60">
+        <v>6.6221360000000002</v>
+      </c>
+      <c r="W60">
+        <v>5.360087</v>
+      </c>
+      <c r="X60">
+        <v>668</v>
+      </c>
+      <c r="Y60">
+        <v>7.3982039999999998</v>
+      </c>
+    </row>
+    <row r="61" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>25</v>
+      </c>
+      <c r="B61" t="s">
+        <v>26</v>
+      </c>
+      <c r="C61" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" t="s">
+        <v>28</v>
+      </c>
+      <c r="E61" t="s">
+        <v>29</v>
+      </c>
+      <c r="F61">
+        <v>303</v>
+      </c>
+      <c r="G61" t="s">
+        <v>42</v>
+      </c>
+      <c r="H61">
+        <v>5170</v>
+      </c>
+      <c r="I61">
+        <v>1.182785</v>
+      </c>
+      <c r="J61">
+        <v>12.0660066</v>
+      </c>
+      <c r="K61">
+        <v>160</v>
+      </c>
+      <c r="L61" t="s">
+        <v>30</v>
+      </c>
+      <c r="M61">
+        <v>3656</v>
+      </c>
+      <c r="N61" t="s">
+        <v>110</v>
+      </c>
+      <c r="O61">
+        <v>6115</v>
+      </c>
+      <c r="P61">
+        <v>597.87408000000005</v>
+      </c>
+      <c r="Q61">
+        <v>303</v>
+      </c>
+      <c r="S61">
+        <v>12.066007000000001</v>
+      </c>
+      <c r="T61">
+        <v>4.9550289999999997</v>
+      </c>
+      <c r="U61">
+        <v>363</v>
+      </c>
+      <c r="V61">
+        <v>5.9362219999999999</v>
+      </c>
+      <c r="W61">
+        <v>10.071624999999999</v>
+      </c>
+      <c r="X61">
+        <v>283</v>
+      </c>
+      <c r="Y61">
+        <v>12.918728</v>
+      </c>
+    </row>
+    <row r="62" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>25</v>
+      </c>
+      <c r="B62" t="s">
+        <v>26</v>
+      </c>
+      <c r="C62" t="s">
+        <v>122</v>
+      </c>
+      <c r="D62" t="s">
+        <v>38</v>
+      </c>
+      <c r="E62" t="s">
+        <v>29</v>
+      </c>
+      <c r="F62">
+        <v>169</v>
+      </c>
+      <c r="G62" t="s">
+        <v>42</v>
+      </c>
+      <c r="H62">
+        <v>5142</v>
+      </c>
+      <c r="I62">
+        <v>1.2957989999999999</v>
+      </c>
+      <c r="J62">
+        <v>29.14792899</v>
+      </c>
+      <c r="K62">
+        <v>160</v>
+      </c>
+      <c r="L62" t="s">
+        <v>30</v>
+      </c>
+      <c r="M62">
+        <v>4926</v>
+      </c>
+      <c r="N62" t="s">
+        <v>110</v>
+      </c>
+      <c r="O62">
+        <v>6663</v>
+      </c>
+      <c r="P62">
+        <v>739.30661899999996</v>
+      </c>
+      <c r="Q62">
+        <v>169</v>
+      </c>
+      <c r="S62">
+        <v>29.147929000000001</v>
+      </c>
+      <c r="T62">
+        <v>2.5363950000000002</v>
+      </c>
+      <c r="U62">
+        <v>210</v>
+      </c>
+      <c r="V62">
+        <v>3.1517330000000001</v>
+      </c>
+      <c r="W62">
+        <v>23.457142999999999</v>
+      </c>
+      <c r="X62">
+        <v>131</v>
+      </c>
+      <c r="Y62">
+        <v>37.603053000000003</v>
+      </c>
+    </row>
+    <row r="63" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>25</v>
+      </c>
+      <c r="B63" t="s">
+        <v>26</v>
+      </c>
+      <c r="C63" t="s">
+        <v>123</v>
+      </c>
+      <c r="D63" t="s">
+        <v>38</v>
+      </c>
+      <c r="E63" t="s">
+        <v>29</v>
+      </c>
+      <c r="F63">
+        <v>196</v>
+      </c>
+      <c r="G63" t="s">
+        <v>42</v>
+      </c>
+      <c r="H63">
+        <v>6373</v>
+      </c>
+      <c r="I63">
+        <v>1.452377</v>
+      </c>
+      <c r="J63">
+        <v>25.10714286</v>
+      </c>
+      <c r="K63">
+        <v>160</v>
+      </c>
+      <c r="L63" t="s">
+        <v>30</v>
+      </c>
+      <c r="M63">
+        <v>4921</v>
+      </c>
+      <c r="N63" t="s">
+        <v>110</v>
+      </c>
+      <c r="O63">
+        <v>9256</v>
+      </c>
+      <c r="P63">
+        <v>531.65514299999995</v>
+      </c>
+      <c r="Q63">
+        <v>196</v>
+      </c>
+      <c r="S63">
+        <v>25.107143000000001</v>
+      </c>
+      <c r="T63">
+        <v>2.1175449999999998</v>
+      </c>
+      <c r="U63">
+        <v>295</v>
+      </c>
+      <c r="V63">
+        <v>3.187122</v>
+      </c>
+      <c r="W63">
+        <v>16.681356000000001</v>
+      </c>
+      <c r="X63">
+        <v>166</v>
+      </c>
+      <c r="Y63">
+        <v>29.644577999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>25</v>
+      </c>
+      <c r="B64" t="s">
+        <v>26</v>
+      </c>
+      <c r="C64" t="s">
+        <v>124</v>
+      </c>
+      <c r="D64" t="s">
+        <v>125</v>
+      </c>
+      <c r="E64" t="s">
+        <v>29</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="K64">
+        <v>160</v>
+      </c>
+      <c r="L64" t="s">
+        <v>30</v>
+      </c>
+      <c r="M64">
+        <v>0</v>
+      </c>
+      <c r="N64" t="s">
+        <v>126</v>
+      </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64">
+        <v>0</v>
+      </c>
+      <c r="U64">
+        <v>0</v>
+      </c>
+      <c r="V64">
+        <v>0</v>
+      </c>
+      <c r="W64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>25</v>
+      </c>
+      <c r="B65" t="s">
+        <v>26</v>
+      </c>
+      <c r="C65" t="s">
+        <v>127</v>
+      </c>
+      <c r="D65" t="s">
+        <v>38</v>
+      </c>
+      <c r="E65" t="s">
+        <v>29</v>
+      </c>
+      <c r="F65">
+        <v>60</v>
+      </c>
+      <c r="G65" t="s">
+        <v>42</v>
+      </c>
+      <c r="H65">
+        <v>4039</v>
+      </c>
+      <c r="I65">
+        <v>1.596187</v>
+      </c>
+      <c r="J65">
+        <v>82.483333329999994</v>
+      </c>
+      <c r="K65">
+        <v>160</v>
+      </c>
+      <c r="L65" t="s">
+        <v>30</v>
+      </c>
+      <c r="M65">
+        <v>4949</v>
+      </c>
+      <c r="N65" t="s">
+        <v>110</v>
+      </c>
+      <c r="O65">
+        <v>6447</v>
+      </c>
+      <c r="P65">
+        <v>767.64386500000001</v>
+      </c>
+      <c r="Q65">
+        <v>60</v>
+      </c>
+      <c r="S65">
+        <v>82.483333000000002</v>
+      </c>
+      <c r="T65">
+        <v>0.93066499999999996</v>
+      </c>
+      <c r="U65">
+        <v>97</v>
+      </c>
+      <c r="V65">
+        <v>1.5045759999999999</v>
+      </c>
+      <c r="W65">
+        <v>51.020619000000003</v>
+      </c>
+      <c r="X65">
+        <v>27</v>
+      </c>
+      <c r="Y65">
+        <v>183.29629600000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>25</v>
+      </c>
+      <c r="B66" t="s">
+        <v>26</v>
+      </c>
+      <c r="C66" t="s">
+        <v>128</v>
+      </c>
+      <c r="D66" t="s">
+        <v>38</v>
+      </c>
+      <c r="E66" t="s">
+        <v>29</v>
+      </c>
+      <c r="F66">
+        <v>409</v>
+      </c>
+      <c r="G66" t="s">
+        <v>42</v>
+      </c>
+      <c r="H66">
+        <v>6062</v>
+      </c>
+      <c r="I66">
+        <v>1.3772679999999999</v>
+      </c>
+      <c r="J66">
+        <v>12.04645477</v>
+      </c>
+      <c r="K66">
+        <v>160</v>
+      </c>
+      <c r="L66" t="s">
+        <v>30</v>
+      </c>
+      <c r="M66">
+        <v>4927</v>
+      </c>
+      <c r="N66" t="s">
+        <v>110</v>
+      </c>
+      <c r="O66">
+        <v>8349</v>
+      </c>
+      <c r="P66">
+        <v>590.13055499999996</v>
+      </c>
+      <c r="Q66">
+        <v>409</v>
+      </c>
+      <c r="S66">
+        <v>12.046455</v>
+      </c>
+      <c r="T66">
+        <v>4.89879</v>
+      </c>
+      <c r="U66">
+        <v>469</v>
+      </c>
+      <c r="V66">
+        <v>5.6174390000000001</v>
+      </c>
+      <c r="W66">
+        <v>10.505330000000001</v>
+      </c>
+      <c r="X66">
+        <v>350</v>
+      </c>
+      <c r="Y66">
+        <v>14.077143</v>
+      </c>
+    </row>
+    <row r="67" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>25</v>
+      </c>
+      <c r="B67" t="s">
+        <v>26</v>
+      </c>
+      <c r="C67" t="s">
+        <v>129</v>
+      </c>
+      <c r="D67" t="s">
+        <v>28</v>
+      </c>
+      <c r="E67" t="s">
+        <v>29</v>
+      </c>
+      <c r="F67">
+        <v>328</v>
+      </c>
+      <c r="G67" t="s">
+        <v>42</v>
+      </c>
+      <c r="H67">
+        <v>3887</v>
+      </c>
+      <c r="I67">
+        <v>1.5346029999999999</v>
+      </c>
+      <c r="J67">
+        <v>11.2195122</v>
+      </c>
+      <c r="K67">
+        <v>160</v>
+      </c>
+      <c r="L67" t="s">
+        <v>30</v>
+      </c>
+      <c r="M67">
+        <v>3680</v>
+      </c>
+      <c r="N67" t="s">
+        <v>110</v>
+      </c>
+      <c r="O67">
+        <v>5965</v>
+      </c>
+      <c r="P67">
+        <v>616.93210399999998</v>
+      </c>
+      <c r="Q67">
+        <v>328</v>
+      </c>
+      <c r="S67">
+        <v>11.219512</v>
+      </c>
+      <c r="T67">
+        <v>5.4987430000000002</v>
+      </c>
+      <c r="U67">
+        <v>388</v>
+      </c>
+      <c r="V67">
+        <v>6.5046099999999996</v>
+      </c>
+      <c r="W67">
+        <v>9.4845360000000003</v>
+      </c>
+      <c r="X67">
+        <v>307</v>
+      </c>
+      <c r="Y67">
+        <v>11.986971</v>
+      </c>
+    </row>
+    <row r="68" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>25</v>
+      </c>
+      <c r="B68" t="s">
+        <v>26</v>
+      </c>
+      <c r="C68" t="s">
+        <v>130</v>
+      </c>
+      <c r="D68" t="s">
+        <v>28</v>
+      </c>
+      <c r="E68" t="s">
+        <v>29</v>
+      </c>
+      <c r="F68">
+        <v>70</v>
+      </c>
+      <c r="G68" t="s">
+        <v>42</v>
+      </c>
+      <c r="H68">
+        <v>2601</v>
+      </c>
+      <c r="I68">
+        <v>1.5809299999999999</v>
+      </c>
+      <c r="J68">
+        <v>70.7</v>
+      </c>
+      <c r="K68">
+        <v>160</v>
+      </c>
+      <c r="L68" t="s">
+        <v>30</v>
+      </c>
+      <c r="M68">
+        <v>4949</v>
+      </c>
+      <c r="N68" t="s">
+        <v>131</v>
+      </c>
+      <c r="O68">
+        <v>4112</v>
+      </c>
+      <c r="P68">
+        <v>1203.5505840000001</v>
+      </c>
+      <c r="Q68">
+        <v>70</v>
+      </c>
+      <c r="S68">
+        <v>70.7</v>
+      </c>
+      <c r="T68">
+        <v>1.7023349999999999</v>
+      </c>
+      <c r="U68">
+        <v>75</v>
+      </c>
+      <c r="V68">
+        <v>1.8239300000000001</v>
+      </c>
+      <c r="W68">
+        <v>65.986666999999997</v>
+      </c>
+      <c r="X68">
+        <v>63</v>
+      </c>
+      <c r="Y68">
+        <v>78.555555999999996</v>
+      </c>
+    </row>
+    <row r="69" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>25</v>
+      </c>
+      <c r="B69" t="s">
+        <v>26</v>
+      </c>
+      <c r="C69" t="s">
+        <v>132</v>
+      </c>
+      <c r="D69" t="s">
+        <v>28</v>
+      </c>
+      <c r="E69" t="s">
+        <v>29</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>0</v>
+      </c>
+      <c r="K69">
+        <v>160</v>
+      </c>
+      <c r="L69" t="s">
+        <v>30</v>
+      </c>
+      <c r="M69">
+        <v>0</v>
+      </c>
+      <c r="N69" t="s">
+        <v>131</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
+      </c>
+      <c r="P69">
+        <v>0</v>
+      </c>
+      <c r="U69">
+        <v>0</v>
+      </c>
+      <c r="V69">
+        <v>0</v>
+      </c>
+      <c r="W69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>25</v>
+      </c>
+      <c r="B70" t="s">
+        <v>26</v>
+      </c>
+      <c r="C70" t="s">
+        <v>133</v>
+      </c>
+      <c r="D70" t="s">
+        <v>134</v>
+      </c>
+      <c r="E70" t="s">
+        <v>29</v>
+      </c>
+      <c r="F70">
+        <v>192</v>
+      </c>
+      <c r="G70" t="s">
+        <v>42</v>
+      </c>
+      <c r="H70">
+        <v>2780</v>
+      </c>
+      <c r="I70">
+        <v>1.5086329999999999</v>
+      </c>
+      <c r="J70">
+        <v>25.651041670000001</v>
+      </c>
+      <c r="K70">
+        <v>160</v>
+      </c>
+      <c r="L70" t="s">
+        <v>30</v>
+      </c>
+      <c r="M70">
+        <v>4925</v>
+      </c>
+      <c r="N70" t="s">
+        <v>60</v>
+      </c>
+      <c r="O70">
+        <v>4194</v>
+      </c>
+      <c r="P70">
+        <v>1174.2966140000001</v>
+      </c>
+      <c r="Q70">
+        <v>192</v>
+      </c>
+      <c r="S70">
+        <v>25.651042</v>
+      </c>
+      <c r="T70">
+        <v>4.5779690000000004</v>
+      </c>
+      <c r="U70">
+        <v>213</v>
+      </c>
+      <c r="V70">
+        <v>5.078684</v>
+      </c>
+      <c r="W70">
+        <v>23.122066</v>
+      </c>
+      <c r="X70">
+        <v>179</v>
+      </c>
+      <c r="Y70">
+        <v>27.513966</v>
+      </c>
+    </row>
+    <row r="71" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>25</v>
+      </c>
+      <c r="B71" t="s">
+        <v>26</v>
+      </c>
+      <c r="C71" t="s">
+        <v>135</v>
+      </c>
+      <c r="D71" t="s">
+        <v>41</v>
+      </c>
+      <c r="E71" t="s">
+        <v>29</v>
+      </c>
+      <c r="F71">
+        <v>111</v>
+      </c>
+      <c r="G71" t="s">
+        <v>42</v>
+      </c>
+      <c r="H71">
+        <v>2689</v>
+      </c>
+      <c r="I71">
+        <v>1.4016360000000001</v>
+      </c>
+      <c r="J71">
+        <v>45.045045049999999</v>
+      </c>
+      <c r="K71">
+        <v>160</v>
+      </c>
+      <c r="L71" t="s">
+        <v>30</v>
+      </c>
+      <c r="M71">
+        <v>5000</v>
+      </c>
+      <c r="N71" t="s">
+        <v>56</v>
+      </c>
+      <c r="O71">
+        <v>3769</v>
+      </c>
+      <c r="P71">
+        <v>1326.6118329999999</v>
+      </c>
+      <c r="Q71">
+        <v>111</v>
+      </c>
+      <c r="S71">
+        <v>45.045045000000002</v>
+      </c>
+      <c r="T71">
+        <v>2.9450780000000001</v>
+      </c>
+      <c r="U71">
+        <v>116</v>
+      </c>
+      <c r="V71">
+        <v>3.0777389999999998</v>
+      </c>
+      <c r="W71">
+        <v>43.103448</v>
+      </c>
+      <c r="X71">
+        <v>90</v>
+      </c>
+      <c r="Y71">
+        <v>55.555556000000003</v>
+      </c>
+    </row>
+    <row r="72" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>25</v>
+      </c>
+      <c r="B72" t="s">
+        <v>26</v>
+      </c>
+      <c r="C72" t="s">
+        <v>135</v>
+      </c>
+      <c r="D72" t="s">
+        <v>41</v>
+      </c>
+      <c r="E72" t="s">
+        <v>29</v>
+      </c>
+      <c r="F72">
+        <v>200</v>
+      </c>
+      <c r="G72" t="s">
+        <v>42</v>
+      </c>
+      <c r="H72">
+        <v>4203</v>
+      </c>
+      <c r="I72">
+        <v>1.6316919999999999</v>
+      </c>
+      <c r="J72">
+        <v>24.84</v>
+      </c>
+      <c r="K72">
+        <v>160</v>
+      </c>
+      <c r="L72" t="s">
+        <v>30</v>
+      </c>
+      <c r="M72">
+        <v>4968</v>
+      </c>
+      <c r="N72" t="s">
+        <v>56</v>
+      </c>
+      <c r="O72">
+        <v>6858</v>
+      </c>
+      <c r="P72">
+        <v>724.409449</v>
+      </c>
+      <c r="Q72">
+        <v>200</v>
+      </c>
+      <c r="S72">
+        <v>24.84</v>
+      </c>
+      <c r="T72">
+        <v>2.9163019999999999</v>
+      </c>
+      <c r="U72">
+        <v>269</v>
+      </c>
+      <c r="V72">
+        <v>3.9224260000000002</v>
+      </c>
+      <c r="W72">
+        <v>18.468401</v>
+      </c>
+      <c r="X72">
+        <v>178</v>
+      </c>
+      <c r="Y72">
+        <v>27.910112000000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>25</v>
+      </c>
+      <c r="B73" t="s">
+        <v>26</v>
+      </c>
+      <c r="C73" t="s">
+        <v>136</v>
+      </c>
+      <c r="D73" t="s">
+        <v>41</v>
+      </c>
+      <c r="E73" t="s">
+        <v>29</v>
+      </c>
+      <c r="F73">
+        <v>241</v>
+      </c>
+      <c r="G73" t="s">
+        <v>42</v>
+      </c>
+      <c r="H73">
+        <v>3334</v>
+      </c>
+      <c r="I73">
+        <v>1.6691659999999999</v>
+      </c>
+      <c r="J73">
+        <v>20.377593359999999</v>
+      </c>
+      <c r="K73">
+        <v>160</v>
+      </c>
+      <c r="L73" t="s">
+        <v>30</v>
+      </c>
+      <c r="M73">
+        <v>4911</v>
+      </c>
+      <c r="N73" t="s">
+        <v>56</v>
+      </c>
+      <c r="O73">
+        <v>5565</v>
+      </c>
+      <c r="P73">
+        <v>882.479784</v>
+      </c>
+      <c r="Q73">
+        <v>241</v>
+      </c>
+      <c r="S73">
+        <v>20.377593000000001</v>
+      </c>
+      <c r="T73">
+        <v>4.3306380000000004</v>
+      </c>
+      <c r="U73">
+        <v>255</v>
+      </c>
+      <c r="V73">
+        <v>4.5822099999999999</v>
+      </c>
+      <c r="W73">
+        <v>19.258824000000001</v>
+      </c>
+      <c r="X73">
+        <v>213</v>
+      </c>
+      <c r="Y73">
+        <v>23.056338</v>
+      </c>
+    </row>
+    <row r="74" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>25</v>
+      </c>
+      <c r="B74" t="s">
+        <v>26</v>
+      </c>
+      <c r="C74" t="s">
+        <v>137</v>
+      </c>
+      <c r="D74" t="s">
+        <v>41</v>
+      </c>
+      <c r="E74" t="s">
+        <v>29</v>
+      </c>
+      <c r="F74">
+        <v>158</v>
+      </c>
+      <c r="G74" t="s">
+        <v>42</v>
+      </c>
+      <c r="H74">
+        <v>3954</v>
+      </c>
+      <c r="I74">
+        <v>1.5048049999999999</v>
+      </c>
+      <c r="J74">
+        <v>31.246835440000002</v>
+      </c>
+      <c r="K74">
+        <v>160</v>
+      </c>
+      <c r="L74" t="s">
+        <v>30</v>
+      </c>
+      <c r="M74">
+        <v>4937</v>
+      </c>
+      <c r="N74" t="s">
+        <v>56</v>
+      </c>
+      <c r="O74">
+        <v>5950</v>
+      </c>
+      <c r="P74">
+        <v>829.74789899999996</v>
+      </c>
+      <c r="Q74">
+        <v>158</v>
+      </c>
+      <c r="S74">
+        <v>31.246835000000001</v>
+      </c>
+      <c r="T74">
+        <v>2.655462</v>
+      </c>
+      <c r="U74">
+        <v>257</v>
+      </c>
+      <c r="V74">
+        <v>4.3193279999999996</v>
+      </c>
+      <c r="W74">
+        <v>19.210117</v>
+      </c>
+      <c r="X74">
+        <v>141</v>
+      </c>
+      <c r="Y74">
+        <v>35.014184</v>
+      </c>
+    </row>
+    <row r="75" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>25</v>
+      </c>
+      <c r="B75" t="s">
+        <v>26</v>
+      </c>
+      <c r="C75" t="s">
+        <v>138</v>
+      </c>
+      <c r="D75" t="s">
+        <v>41</v>
+      </c>
+      <c r="E75" t="s">
+        <v>29</v>
+      </c>
+      <c r="F75">
+        <v>166</v>
+      </c>
+      <c r="G75" t="s">
+        <v>42</v>
+      </c>
+      <c r="H75">
+        <v>4616</v>
+      </c>
+      <c r="I75">
+        <v>1.666161</v>
+      </c>
+      <c r="J75">
+        <v>29.753012049999999</v>
+      </c>
+      <c r="K75">
+        <v>160</v>
+      </c>
+      <c r="L75" t="s">
+        <v>30</v>
+      </c>
+      <c r="M75">
+        <v>4939</v>
+      </c>
+      <c r="N75" t="s">
+        <v>56</v>
+      </c>
+      <c r="O75">
+        <v>7691</v>
+      </c>
+      <c r="P75">
+        <v>642.17917</v>
+      </c>
+      <c r="Q75">
+        <v>166</v>
+      </c>
+      <c r="S75">
+        <v>29.753011999999998</v>
+      </c>
+      <c r="T75">
+        <v>2.1583670000000001</v>
+      </c>
+      <c r="U75">
+        <v>242</v>
+      </c>
+      <c r="V75">
+        <v>3.1465350000000001</v>
+      </c>
+      <c r="W75">
+        <v>20.409091</v>
+      </c>
+      <c r="X75">
+        <v>159</v>
+      </c>
+      <c r="Y75">
+        <v>31.062892999999999</v>
+      </c>
+    </row>
+    <row r="76" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>25</v>
+      </c>
+      <c r="B76" t="s">
+        <v>26</v>
+      </c>
+      <c r="C76" t="s">
+        <v>139</v>
+      </c>
+      <c r="D76" t="s">
+        <v>28</v>
+      </c>
+      <c r="E76" t="s">
+        <v>29</v>
+      </c>
+      <c r="F76">
+        <v>113</v>
+      </c>
+      <c r="G76" t="s">
+        <v>42</v>
+      </c>
+      <c r="H76">
+        <v>3444</v>
+      </c>
+      <c r="I76">
+        <v>1.5383279999999999</v>
+      </c>
+      <c r="J76">
+        <v>43.707964599999997</v>
+      </c>
+      <c r="K76">
+        <v>160</v>
+      </c>
+      <c r="L76" t="s">
+        <v>30</v>
+      </c>
+      <c r="M76">
+        <v>4939</v>
+      </c>
+      <c r="N76" t="s">
+        <v>56</v>
+      </c>
+      <c r="O76">
+        <v>5298</v>
+      </c>
+      <c r="P76">
+        <v>932.23858099999995</v>
+      </c>
+      <c r="Q76">
+        <v>113</v>
+      </c>
+      <c r="S76">
+        <v>43.707965000000002</v>
+      </c>
+      <c r="T76">
+        <v>2.1328800000000001</v>
+      </c>
+      <c r="U76">
+        <v>131</v>
+      </c>
+      <c r="V76">
+        <v>2.4726309999999998</v>
+      </c>
+      <c r="W76">
+        <v>37.702289999999998</v>
+      </c>
+      <c r="X76">
+        <v>100</v>
+      </c>
+      <c r="Y76">
+        <v>49.39</v>
+      </c>
+    </row>
+    <row r="77" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>25</v>
+      </c>
+      <c r="B77" t="s">
+        <v>26</v>
+      </c>
+      <c r="C77" t="s">
+        <v>140</v>
+      </c>
+      <c r="D77" t="s">
+        <v>28</v>
+      </c>
+      <c r="E77" t="s">
+        <v>29</v>
+      </c>
+      <c r="F77">
+        <v>85</v>
+      </c>
+      <c r="G77" t="s">
+        <v>42</v>
+      </c>
+      <c r="H77">
+        <v>3376</v>
+      </c>
+      <c r="I77">
+        <v>1.3939569999999999</v>
+      </c>
+      <c r="J77">
+        <v>58.047058819999997</v>
+      </c>
+      <c r="K77">
+        <v>160</v>
+      </c>
+      <c r="L77" t="s">
+        <v>30</v>
+      </c>
+      <c r="M77">
+        <v>4934</v>
+      </c>
+      <c r="N77" t="s">
+        <v>56</v>
+      </c>
+      <c r="O77">
+        <v>4706</v>
+      </c>
+      <c r="P77">
+        <v>1048.448789</v>
+      </c>
+      <c r="Q77">
+        <v>85</v>
+      </c>
+      <c r="S77">
+        <v>58.047058999999997</v>
+      </c>
+      <c r="T77">
+        <v>1.8062050000000001</v>
+      </c>
+      <c r="U77">
+        <v>111</v>
+      </c>
+      <c r="V77">
+        <v>2.3586909999999999</v>
+      </c>
+      <c r="W77">
+        <v>44.450449999999996</v>
+      </c>
+      <c r="X77">
+        <v>81</v>
+      </c>
+      <c r="Y77">
+        <v>60.913580000000003</v>
+      </c>
+    </row>
+    <row r="78" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>25</v>
+      </c>
+      <c r="B78" t="s">
+        <v>26</v>
+      </c>
+      <c r="C78" t="s">
+        <v>141</v>
+      </c>
+      <c r="D78" t="s">
+        <v>41</v>
+      </c>
+      <c r="E78" t="s">
+        <v>29</v>
+      </c>
+      <c r="F78">
+        <v>144</v>
+      </c>
+      <c r="G78" t="s">
+        <v>42</v>
+      </c>
+      <c r="H78">
+        <v>3178</v>
+      </c>
+      <c r="I78">
+        <v>1.7702960000000001</v>
+      </c>
+      <c r="J78">
+        <v>34.284722219999999</v>
+      </c>
+      <c r="K78">
+        <v>160</v>
+      </c>
+      <c r="L78" t="s">
+        <v>30</v>
+      </c>
+      <c r="M78">
+        <v>4937</v>
+      </c>
+      <c r="N78" t="s">
+        <v>142</v>
+      </c>
+      <c r="O78">
+        <v>5626</v>
+      </c>
+      <c r="P78">
+        <v>877.53288299999997</v>
+      </c>
+      <c r="Q78">
+        <v>144</v>
+      </c>
+      <c r="S78">
+        <v>34.284722000000002</v>
+      </c>
+      <c r="T78">
+        <v>2.559545</v>
+      </c>
+      <c r="U78">
+        <v>203</v>
+      </c>
+      <c r="V78">
+        <v>3.608247</v>
+      </c>
+      <c r="W78">
+        <v>24.320197</v>
+      </c>
+      <c r="X78">
+        <v>48</v>
+      </c>
+      <c r="Y78">
+        <v>102.854167</v>
+      </c>
+    </row>
+    <row r="79" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>25</v>
+      </c>
+      <c r="B79" t="s">
+        <v>26</v>
+      </c>
+      <c r="C79" t="s">
+        <v>143</v>
+      </c>
+      <c r="D79" t="s">
+        <v>41</v>
+      </c>
+      <c r="E79" t="s">
+        <v>29</v>
+      </c>
+      <c r="F79">
+        <v>109</v>
+      </c>
+      <c r="G79" t="s">
+        <v>42</v>
+      </c>
+      <c r="H79">
+        <v>2835</v>
+      </c>
+      <c r="I79">
+        <v>2.1527340000000001</v>
+      </c>
+      <c r="J79">
+        <v>44.715596329999997</v>
+      </c>
+      <c r="K79">
+        <v>160</v>
+      </c>
+      <c r="L79" t="s">
+        <v>30</v>
+      </c>
+      <c r="M79">
+        <v>4874</v>
+      </c>
+      <c r="N79" t="s">
+        <v>56</v>
+      </c>
+      <c r="O79">
+        <v>6103</v>
+      </c>
+      <c r="P79">
+        <v>798.62362800000005</v>
+      </c>
+      <c r="Q79">
+        <v>109</v>
+      </c>
+      <c r="S79">
+        <v>44.715595999999998</v>
+      </c>
+      <c r="T79">
+        <v>1.7860069999999999</v>
+      </c>
+      <c r="U79">
+        <v>150</v>
+      </c>
+      <c r="V79">
+        <v>2.457808</v>
+      </c>
+      <c r="W79">
+        <v>32.493333</v>
+      </c>
+      <c r="X79">
+        <v>88</v>
+      </c>
+      <c r="Y79">
+        <v>55.386364</v>
+      </c>
+    </row>
+    <row r="80" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>25</v>
+      </c>
+      <c r="B80" t="s">
+        <v>26</v>
+      </c>
+      <c r="C80" t="s">
+        <v>144</v>
+      </c>
+      <c r="D80" t="s">
+        <v>41</v>
+      </c>
+      <c r="E80" t="s">
+        <v>29</v>
+      </c>
+      <c r="F80">
+        <v>218</v>
+      </c>
+      <c r="G80" t="s">
+        <v>42</v>
+      </c>
+      <c r="H80">
+        <v>2954</v>
+      </c>
+      <c r="I80">
+        <v>1.6181449999999999</v>
+      </c>
+      <c r="J80">
+        <v>22.605504589999999</v>
+      </c>
+      <c r="K80">
+        <v>160</v>
+      </c>
+      <c r="L80" t="s">
+        <v>30</v>
+      </c>
+      <c r="M80">
+        <v>4928</v>
+      </c>
+      <c r="N80" t="s">
+        <v>56</v>
+      </c>
+      <c r="O80">
+        <v>4780</v>
+      </c>
+      <c r="P80">
+        <v>1030.9623429999999</v>
+      </c>
+      <c r="Q80">
+        <v>218</v>
+      </c>
+      <c r="S80">
+        <v>22.605505000000001</v>
+      </c>
+      <c r="T80">
+        <v>4.5606689999999999</v>
+      </c>
+      <c r="U80">
+        <v>232</v>
+      </c>
+      <c r="V80">
+        <v>4.8535560000000002</v>
+      </c>
+      <c r="W80">
+        <v>21.241378999999998</v>
+      </c>
+      <c r="X80">
+        <v>199</v>
+      </c>
+      <c r="Y80">
+        <v>24.763819000000002</v>
+      </c>
+    </row>
+    <row r="81" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>25</v>
+      </c>
+      <c r="B81" t="s">
+        <v>26</v>
+      </c>
+      <c r="C81" t="s">
+        <v>145</v>
+      </c>
+      <c r="D81" t="s">
+        <v>41</v>
+      </c>
+      <c r="E81" t="s">
+        <v>29</v>
+      </c>
+      <c r="F81">
+        <v>417</v>
+      </c>
+      <c r="G81" t="s">
+        <v>42</v>
+      </c>
+      <c r="H81">
+        <v>6246</v>
+      </c>
+      <c r="I81">
+        <v>1.5073650000000001</v>
+      </c>
+      <c r="J81">
+        <v>11.83932854</v>
+      </c>
+      <c r="K81">
+        <v>160</v>
+      </c>
+      <c r="L81" t="s">
+        <v>30</v>
+      </c>
+      <c r="M81">
+        <v>4937</v>
+      </c>
+      <c r="N81" t="s">
+        <v>56</v>
+      </c>
+      <c r="O81">
+        <v>9415</v>
+      </c>
+      <c r="P81">
+        <v>524.37599599999999</v>
+      </c>
+      <c r="Q81">
+        <v>417</v>
+      </c>
+      <c r="S81">
+        <v>11.839328999999999</v>
+      </c>
+      <c r="T81">
+        <v>4.4291029999999996</v>
+      </c>
+      <c r="U81">
+        <v>492</v>
+      </c>
+      <c r="V81">
+        <v>5.2257040000000003</v>
+      </c>
+      <c r="W81">
+        <v>10.034553000000001</v>
+      </c>
+      <c r="X81">
+        <v>386</v>
+      </c>
+      <c r="Y81">
+        <v>12.790155</v>
+      </c>
+    </row>
+    <row r="82" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>25</v>
+      </c>
+      <c r="B82" t="s">
+        <v>26</v>
+      </c>
+      <c r="C82" t="s">
+        <v>146</v>
+      </c>
+      <c r="D82" t="s">
+        <v>41</v>
+      </c>
+      <c r="E82" t="s">
+        <v>29</v>
+      </c>
+      <c r="F82">
+        <v>592</v>
+      </c>
+      <c r="G82" t="s">
+        <v>42</v>
+      </c>
+      <c r="H82">
+        <v>4816</v>
+      </c>
+      <c r="I82">
+        <v>1.5517030000000001</v>
+      </c>
+      <c r="J82">
+        <v>8.4054054100000002</v>
+      </c>
+      <c r="K82">
+        <v>160</v>
+      </c>
+      <c r="L82" t="s">
+        <v>30</v>
+      </c>
+      <c r="M82">
+        <v>4976</v>
+      </c>
+      <c r="N82" t="s">
+        <v>56</v>
+      </c>
+      <c r="O82">
+        <v>7473</v>
+      </c>
+      <c r="P82">
+        <v>665.86377600000003</v>
+      </c>
+      <c r="Q82">
+        <v>592</v>
+      </c>
+      <c r="S82">
+        <v>8.405405</v>
+      </c>
+      <c r="T82">
+        <v>7.9218520000000003</v>
+      </c>
+      <c r="U82">
+        <v>622</v>
+      </c>
+      <c r="V82">
+        <v>8.3232970000000002</v>
+      </c>
+      <c r="W82">
+        <v>8</v>
+      </c>
+      <c r="X82">
+        <v>525</v>
+      </c>
+      <c r="Y82">
+        <v>9.4780949999999997</v>
+      </c>
+    </row>
+    <row r="83" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>25</v>
+      </c>
+      <c r="B83" t="s">
+        <v>26</v>
+      </c>
+      <c r="C83" t="s">
+        <v>132</v>
+      </c>
+      <c r="D83" t="s">
+        <v>28</v>
+      </c>
+      <c r="E83" t="s">
+        <v>29</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <v>160</v>
+      </c>
+      <c r="L83" t="s">
+        <v>30</v>
+      </c>
+      <c r="M83">
+        <v>0</v>
+      </c>
+      <c r="N83" t="s">
+        <v>131</v>
+      </c>
+      <c r="O83">
+        <v>0</v>
+      </c>
+      <c r="P83">
+        <v>0</v>
+      </c>
+      <c r="U83">
+        <v>0</v>
+      </c>
+      <c r="V83">
+        <v>0</v>
+      </c>
+      <c r="W83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>25</v>
+      </c>
+      <c r="B84" t="s">
+        <v>26</v>
+      </c>
+      <c r="C84" t="s">
+        <v>130</v>
+      </c>
+      <c r="D84" t="s">
+        <v>28</v>
+      </c>
+      <c r="E84" t="s">
+        <v>29</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84">
+        <v>0</v>
+      </c>
+      <c r="K84">
+        <v>160</v>
+      </c>
+      <c r="L84" t="s">
+        <v>30</v>
+      </c>
+      <c r="M84">
+        <v>0</v>
+      </c>
+      <c r="N84" t="s">
+        <v>131</v>
+      </c>
+      <c r="O84">
+        <v>0</v>
+      </c>
+      <c r="P84">
+        <v>0</v>
+      </c>
+      <c r="U84">
+        <v>0</v>
+      </c>
+      <c r="V84">
+        <v>0</v>
+      </c>
+      <c r="W84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>25</v>
+      </c>
+      <c r="B85" t="s">
+        <v>26</v>
+      </c>
+      <c r="C85" t="s">
+        <v>147</v>
+      </c>
+      <c r="D85" t="s">
+        <v>41</v>
+      </c>
+      <c r="E85" t="s">
+        <v>29</v>
+      </c>
+      <c r="F85">
+        <v>216</v>
+      </c>
+      <c r="G85" t="s">
+        <v>42</v>
+      </c>
+      <c r="H85">
+        <v>4966</v>
+      </c>
+      <c r="I85">
+        <v>1.353202</v>
+      </c>
+      <c r="J85">
+        <v>23</v>
+      </c>
+      <c r="K85">
+        <v>160</v>
+      </c>
+      <c r="L85" t="s">
+        <v>30</v>
+      </c>
+      <c r="M85">
+        <v>4968</v>
+      </c>
+      <c r="N85" t="s">
+        <v>56</v>
+      </c>
+      <c r="O85">
+        <v>6720</v>
+      </c>
+      <c r="P85">
+        <v>739.28571399999998</v>
+      </c>
+      <c r="Q85">
+        <v>216</v>
+      </c>
+      <c r="S85">
+        <v>23</v>
+      </c>
+      <c r="T85">
+        <v>3.214286</v>
+      </c>
+      <c r="U85">
+        <v>236</v>
+      </c>
+      <c r="V85">
+        <v>3.5119050000000001</v>
+      </c>
+      <c r="W85">
+        <v>21.050847000000001</v>
+      </c>
+      <c r="X85">
+        <v>149</v>
+      </c>
+      <c r="Y85">
+        <v>33.342281999999997</v>
+      </c>
+    </row>
+    <row r="86" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>25</v>
+      </c>
+      <c r="B86" t="s">
+        <v>26</v>
+      </c>
+      <c r="C86" t="s">
+        <v>148</v>
+      </c>
+      <c r="D86" t="s">
+        <v>41</v>
+      </c>
+      <c r="E86" t="s">
+        <v>29</v>
+      </c>
+      <c r="F86">
+        <v>411</v>
+      </c>
+      <c r="G86" t="s">
+        <v>42</v>
+      </c>
+      <c r="H86">
+        <v>5418</v>
+      </c>
+      <c r="I86">
+        <v>1.6035440000000001</v>
+      </c>
+      <c r="J86">
+        <v>11.958637469999999</v>
+      </c>
+      <c r="K86">
+        <v>160</v>
+      </c>
+      <c r="L86" t="s">
+        <v>30</v>
+      </c>
+      <c r="M86">
+        <v>4915</v>
+      </c>
+      <c r="N86" t="s">
+        <v>56</v>
+      </c>
+      <c r="O86">
+        <v>8688</v>
+      </c>
+      <c r="P86">
+        <v>565.72283600000003</v>
+      </c>
+      <c r="Q86">
+        <v>411</v>
+      </c>
+      <c r="S86">
+        <v>11.958637</v>
+      </c>
+      <c r="T86">
+        <v>4.7306629999999998</v>
+      </c>
+      <c r="U86">
+        <v>488</v>
+      </c>
+      <c r="V86">
+        <v>5.616943</v>
+      </c>
+      <c r="W86">
+        <v>10.071721</v>
+      </c>
+      <c r="X86">
+        <v>363</v>
+      </c>
+      <c r="Y86">
+        <v>13.539944999999999</v>
+      </c>
+    </row>
+    <row r="87" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>25</v>
+      </c>
+      <c r="B87" t="s">
+        <v>26</v>
+      </c>
+      <c r="C87" t="s">
+        <v>149</v>
+      </c>
+      <c r="D87" t="s">
+        <v>41</v>
+      </c>
+      <c r="E87" t="s">
+        <v>29</v>
+      </c>
+      <c r="F87">
+        <v>223</v>
+      </c>
+      <c r="G87" t="s">
+        <v>42</v>
+      </c>
+      <c r="H87">
+        <v>3378</v>
+      </c>
+      <c r="I87">
+        <v>1.595915</v>
+      </c>
+      <c r="J87">
+        <v>22.32735426</v>
+      </c>
+      <c r="K87">
+        <v>160</v>
+      </c>
+      <c r="L87" t="s">
+        <v>30</v>
+      </c>
+      <c r="M87">
+        <v>4979</v>
+      </c>
+      <c r="N87" t="s">
+        <v>56</v>
+      </c>
+      <c r="O87">
+        <v>5391</v>
+      </c>
+      <c r="P87">
+        <v>923.57633099999998</v>
+      </c>
+      <c r="Q87">
+        <v>223</v>
+      </c>
+      <c r="S87">
+        <v>22.327354</v>
+      </c>
+      <c r="T87">
+        <v>4.1365239999999996</v>
+      </c>
+      <c r="U87">
+        <v>249</v>
+      </c>
+      <c r="V87">
+        <v>4.6188089999999997</v>
+      </c>
+      <c r="W87">
+        <v>19.995984</v>
+      </c>
+      <c r="X87">
+        <v>204</v>
+      </c>
+      <c r="Y87">
+        <v>24.406863000000001</v>
+      </c>
+    </row>
+    <row r="88" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>25</v>
+      </c>
+      <c r="B88" t="s">
+        <v>26</v>
+      </c>
+      <c r="C88" t="s">
+        <v>150</v>
+      </c>
+      <c r="D88" t="s">
+        <v>41</v>
+      </c>
+      <c r="E88" t="s">
+        <v>29</v>
+      </c>
+      <c r="F88">
+        <v>141</v>
+      </c>
+      <c r="G88" t="s">
+        <v>42</v>
+      </c>
+      <c r="H88">
+        <v>5977</v>
+      </c>
+      <c r="I88">
+        <v>1.228375</v>
+      </c>
+      <c r="J88">
+        <v>35.361702129999998</v>
+      </c>
+      <c r="K88">
+        <v>160</v>
+      </c>
+      <c r="L88" t="s">
+        <v>30</v>
+      </c>
+      <c r="M88">
+        <v>4986</v>
+      </c>
+      <c r="N88" t="s">
+        <v>56</v>
+      </c>
+      <c r="O88">
+        <v>7342</v>
+      </c>
+      <c r="P88">
+        <v>679.10650999999996</v>
+      </c>
+      <c r="Q88">
+        <v>141</v>
+      </c>
+      <c r="S88">
+        <v>35.361702000000001</v>
+      </c>
+      <c r="T88">
+        <v>1.920458</v>
+      </c>
+      <c r="U88">
+        <v>210</v>
+      </c>
+      <c r="V88">
+        <v>2.8602560000000001</v>
+      </c>
+      <c r="W88">
+        <v>23.742857000000001</v>
+      </c>
+      <c r="X88">
+        <v>129</v>
+      </c>
+      <c r="Y88">
+        <v>38.651162999999997</v>
+      </c>
+    </row>
+    <row r="89" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>25</v>
+      </c>
+      <c r="B89" t="s">
+        <v>26</v>
+      </c>
+      <c r="C89" t="s">
+        <v>151</v>
+      </c>
+      <c r="D89" t="s">
+        <v>28</v>
+      </c>
+      <c r="E89" t="s">
+        <v>29</v>
+      </c>
+      <c r="F89">
+        <v>150</v>
+      </c>
+      <c r="G89" t="s">
+        <v>42</v>
+      </c>
+      <c r="H89">
+        <v>3816</v>
+      </c>
+      <c r="I89">
+        <v>1.601939</v>
+      </c>
+      <c r="J89">
+        <v>33.18</v>
+      </c>
+      <c r="K89">
+        <v>160</v>
+      </c>
+      <c r="L89" t="s">
+        <v>30</v>
+      </c>
+      <c r="M89">
+        <v>4977</v>
+      </c>
+      <c r="N89" t="s">
+        <v>56</v>
+      </c>
+      <c r="O89">
+        <v>6113</v>
+      </c>
+      <c r="P89">
+        <v>814.16652999999997</v>
+      </c>
+      <c r="Q89">
+        <v>150</v>
+      </c>
+      <c r="S89">
+        <v>33.18</v>
+      </c>
+      <c r="T89">
+        <v>2.4537870000000002</v>
+      </c>
+      <c r="U89">
+        <v>180</v>
+      </c>
+      <c r="V89">
+        <v>2.9445440000000001</v>
+      </c>
+      <c r="W89">
+        <v>27.65</v>
+      </c>
+      <c r="X89">
+        <v>138</v>
+      </c>
+      <c r="Y89">
+        <v>36.065216999999997</v>
+      </c>
+    </row>
+    <row r="90" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>25</v>
+      </c>
+      <c r="B90" t="s">
+        <v>26</v>
+      </c>
+      <c r="C90" t="s">
+        <v>152</v>
+      </c>
+      <c r="D90" t="s">
+        <v>28</v>
+      </c>
+      <c r="E90" t="s">
+        <v>29</v>
+      </c>
+      <c r="F90">
+        <v>79</v>
+      </c>
+      <c r="G90" t="s">
+        <v>42</v>
+      </c>
+      <c r="H90">
+        <v>2278</v>
+      </c>
+      <c r="I90">
+        <v>1.4231780000000001</v>
+      </c>
+      <c r="J90">
+        <v>62.936708860000003</v>
+      </c>
+      <c r="K90">
+        <v>160</v>
+      </c>
+      <c r="L90" t="s">
+        <v>30</v>
+      </c>
+      <c r="M90">
+        <v>4972</v>
+      </c>
+      <c r="N90" t="s">
+        <v>56</v>
+      </c>
+      <c r="O90">
+        <v>3242</v>
+      </c>
+      <c r="P90">
+        <v>1533.6212210000001</v>
+      </c>
+      <c r="Q90">
+        <v>79</v>
+      </c>
+      <c r="S90">
+        <v>62.936709</v>
+      </c>
+      <c r="T90">
+        <v>2.4367670000000001</v>
+      </c>
+      <c r="U90">
+        <v>92</v>
+      </c>
+      <c r="V90">
+        <v>2.8377539999999999</v>
+      </c>
+      <c r="W90">
+        <v>54.043478</v>
+      </c>
+      <c r="X90">
+        <v>70</v>
+      </c>
+      <c r="Y90">
+        <v>71.028570999999999</v>
+      </c>
+    </row>
+    <row r="91" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>25</v>
+      </c>
+      <c r="B91" t="s">
+        <v>26</v>
+      </c>
+      <c r="C91" t="s">
+        <v>153</v>
+      </c>
+      <c r="D91" t="s">
+        <v>41</v>
+      </c>
+      <c r="E91" t="s">
+        <v>29</v>
+      </c>
+      <c r="F91">
+        <v>127</v>
+      </c>
+      <c r="G91" t="s">
+        <v>42</v>
+      </c>
+      <c r="H91">
+        <v>2985</v>
+      </c>
+      <c r="I91">
+        <v>1.4335009999999999</v>
+      </c>
+      <c r="J91">
+        <v>38.944881889999998</v>
+      </c>
+      <c r="K91">
+        <v>160</v>
+      </c>
+      <c r="L91" t="s">
+        <v>30</v>
+      </c>
+      <c r="M91">
+        <v>4946</v>
+      </c>
+      <c r="N91" t="s">
+        <v>56</v>
+      </c>
+      <c r="O91">
+        <v>4279</v>
+      </c>
+      <c r="P91">
+        <v>1155.8775410000001</v>
+      </c>
+      <c r="Q91">
+        <v>127</v>
+      </c>
+      <c r="S91">
+        <v>38.944882</v>
+      </c>
+      <c r="T91">
+        <v>2.9679829999999998</v>
+      </c>
+      <c r="U91">
+        <v>139</v>
+      </c>
+      <c r="V91">
+        <v>3.2484229999999998</v>
+      </c>
+      <c r="W91">
+        <v>35.582734000000002</v>
+      </c>
+      <c r="X91">
+        <v>113</v>
+      </c>
+      <c r="Y91">
+        <v>43.769911999999998</v>
+      </c>
+    </row>
+    <row r="92" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>25</v>
+      </c>
+      <c r="B92" t="s">
+        <v>26</v>
+      </c>
+      <c r="C92" t="s">
+        <v>154</v>
+      </c>
+      <c r="D92" t="s">
+        <v>41</v>
+      </c>
+      <c r="E92" t="s">
+        <v>29</v>
+      </c>
+      <c r="F92">
+        <v>142</v>
+      </c>
+      <c r="G92" t="s">
+        <v>42</v>
+      </c>
+      <c r="H92">
+        <v>3096</v>
+      </c>
+      <c r="I92">
+        <v>1.5329459999999999</v>
+      </c>
+      <c r="J92">
+        <v>35.112676059999998</v>
+      </c>
+      <c r="K92">
+        <v>160</v>
+      </c>
+      <c r="L92" t="s">
+        <v>30</v>
+      </c>
+      <c r="M92">
+        <v>4986</v>
+      </c>
+      <c r="N92" t="s">
+        <v>56</v>
+      </c>
+      <c r="O92">
+        <v>4746</v>
+      </c>
+      <c r="P92">
+        <v>1050.5689</v>
+      </c>
+      <c r="Q92">
+        <v>142</v>
+      </c>
+      <c r="S92">
+        <v>35.112676</v>
+      </c>
+      <c r="T92">
+        <v>2.9919929999999999</v>
+      </c>
+      <c r="U92">
+        <v>166</v>
+      </c>
+      <c r="V92">
+        <v>3.4976820000000002</v>
+      </c>
+      <c r="W92">
+        <v>30.036145000000001</v>
+      </c>
+      <c r="X92">
+        <v>132</v>
+      </c>
+      <c r="Y92">
+        <v>37.772727000000003</v>
+      </c>
+    </row>
+    <row r="93" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>25</v>
+      </c>
+      <c r="B93" t="s">
+        <v>26</v>
+      </c>
+      <c r="C93" t="s">
+        <v>155</v>
+      </c>
+      <c r="D93" t="s">
+        <v>41</v>
+      </c>
+      <c r="E93" t="s">
+        <v>29</v>
+      </c>
+      <c r="F93">
+        <v>153</v>
+      </c>
+      <c r="G93" t="s">
+        <v>42</v>
+      </c>
+      <c r="H93">
+        <v>3237</v>
+      </c>
+      <c r="I93">
+        <v>1.8115540000000001</v>
+      </c>
+      <c r="J93">
+        <v>32.516339870000003</v>
+      </c>
+      <c r="K93">
+        <v>160</v>
+      </c>
+      <c r="L93" t="s">
+        <v>30</v>
+      </c>
+      <c r="M93">
+        <v>4975</v>
+      </c>
+      <c r="N93" t="s">
+        <v>56</v>
+      </c>
+      <c r="O93">
+        <v>5864</v>
+      </c>
+      <c r="P93">
+        <v>848.39699900000005</v>
+      </c>
+      <c r="Q93">
+        <v>153</v>
+      </c>
+      <c r="S93">
+        <v>32.51634</v>
+      </c>
+      <c r="T93">
+        <v>2.6091410000000002</v>
+      </c>
+      <c r="U93">
+        <v>184</v>
+      </c>
+      <c r="V93">
+        <v>3.1377899999999999</v>
+      </c>
+      <c r="W93">
+        <v>27.038042999999998</v>
+      </c>
+      <c r="X93">
+        <v>148</v>
+      </c>
+      <c r="Y93">
+        <v>33.614865000000002</v>
+      </c>
+    </row>
+    <row r="94" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>25</v>
+      </c>
+      <c r="B94" t="s">
+        <v>26</v>
+      </c>
+      <c r="C94" t="s">
+        <v>156</v>
+      </c>
+      <c r="D94" t="s">
+        <v>41</v>
+      </c>
+      <c r="E94" t="s">
+        <v>29</v>
+      </c>
+      <c r="F94">
+        <v>137</v>
+      </c>
+      <c r="G94" t="s">
+        <v>42</v>
+      </c>
+      <c r="H94">
+        <v>5610</v>
+      </c>
+      <c r="I94">
+        <v>1.5240640000000001</v>
+      </c>
+      <c r="J94">
+        <v>36.306569340000003</v>
+      </c>
+      <c r="K94">
+        <v>160</v>
+      </c>
+      <c r="L94" t="s">
+        <v>30</v>
+      </c>
+      <c r="M94">
+        <v>4974</v>
+      </c>
+      <c r="N94" t="s">
+        <v>56</v>
+      </c>
+      <c r="O94">
+        <v>8550</v>
+      </c>
+      <c r="P94">
+        <v>581.75438599999995</v>
+      </c>
+      <c r="Q94">
+        <v>137</v>
+      </c>
+      <c r="S94">
+        <v>36.306569000000003</v>
+      </c>
+      <c r="T94">
+        <v>1.602339</v>
+      </c>
+      <c r="U94">
+        <v>186</v>
+      </c>
+      <c r="V94">
+        <v>2.1754389999999999</v>
+      </c>
+      <c r="W94">
+        <v>26.741935000000002</v>
+      </c>
+      <c r="X94">
+        <v>127</v>
+      </c>
+      <c r="Y94">
+        <v>39.165354000000001</v>
+      </c>
+    </row>
+    <row r="95" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>25</v>
+      </c>
+      <c r="B95" t="s">
+        <v>26</v>
+      </c>
+      <c r="C95" t="s">
+        <v>157</v>
+      </c>
+      <c r="D95" t="s">
+        <v>41</v>
+      </c>
+      <c r="E95" t="s">
+        <v>29</v>
+      </c>
+      <c r="F95">
+        <v>106</v>
+      </c>
+      <c r="G95" t="s">
+        <v>42</v>
+      </c>
+      <c r="H95">
+        <v>2393</v>
+      </c>
+      <c r="I95">
+        <v>1.4860009999999999</v>
+      </c>
+      <c r="J95">
+        <v>46.716981130000001</v>
+      </c>
+      <c r="K95">
+        <v>160</v>
+      </c>
+      <c r="L95" t="s">
+        <v>30</v>
+      </c>
+      <c r="M95">
+        <v>4952</v>
+      </c>
+      <c r="N95" t="s">
+        <v>158</v>
+      </c>
+      <c r="O95">
+        <v>3556</v>
+      </c>
+      <c r="P95">
+        <v>1392.575928</v>
+      </c>
+      <c r="Q95">
+        <v>106</v>
+      </c>
+      <c r="S95">
+        <v>46.716980999999997</v>
+      </c>
+      <c r="T95">
+        <v>2.980877</v>
+      </c>
+      <c r="U95">
+        <v>115</v>
+      </c>
+      <c r="V95">
+        <v>3.2339709999999999</v>
+      </c>
+      <c r="W95">
+        <v>43.060870000000001</v>
+      </c>
+      <c r="X95">
+        <v>30</v>
+      </c>
+      <c r="Y95">
+        <v>165.066667</v>
+      </c>
+    </row>
+    <row r="96" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>25</v>
+      </c>
+      <c r="B96" t="s">
+        <v>26</v>
+      </c>
+      <c r="C96" t="s">
+        <v>159</v>
+      </c>
+      <c r="D96" t="s">
+        <v>41</v>
+      </c>
+      <c r="E96" t="s">
+        <v>29</v>
+      </c>
+      <c r="F96">
+        <v>128</v>
+      </c>
+      <c r="G96" t="s">
+        <v>42</v>
+      </c>
+      <c r="H96">
+        <v>3059</v>
+      </c>
+      <c r="I96">
+        <v>1.613599</v>
+      </c>
+      <c r="J96">
+        <v>38.90625</v>
+      </c>
+      <c r="K96">
+        <v>160</v>
+      </c>
+      <c r="L96" t="s">
+        <v>30</v>
+      </c>
+      <c r="M96">
+        <v>4980</v>
+      </c>
+      <c r="N96" t="s">
+        <v>158</v>
+      </c>
+      <c r="O96">
+        <v>4936</v>
+      </c>
+      <c r="P96">
+        <v>1008.9141</v>
+      </c>
+      <c r="Q96">
+        <v>128</v>
+      </c>
+      <c r="S96">
+        <v>38.90625</v>
+      </c>
+      <c r="T96">
+        <v>2.5931929999999999</v>
+      </c>
+      <c r="U96">
+        <v>144</v>
+      </c>
+      <c r="V96">
+        <v>2.9173420000000001</v>
+      </c>
+      <c r="W96">
+        <v>34.583333000000003</v>
+      </c>
+      <c r="X96">
+        <v>72</v>
+      </c>
+      <c r="Y96">
+        <v>69.166667000000004</v>
+      </c>
+    </row>
+    <row r="97" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>25</v>
+      </c>
+      <c r="B97" t="s">
+        <v>26</v>
+      </c>
+      <c r="C97" t="s">
+        <v>160</v>
+      </c>
+      <c r="D97" t="s">
+        <v>41</v>
+      </c>
+      <c r="E97" t="s">
+        <v>29</v>
+      </c>
+      <c r="F97">
+        <v>150</v>
+      </c>
+      <c r="G97" t="s">
+        <v>42</v>
+      </c>
+      <c r="H97">
+        <v>2991</v>
+      </c>
+      <c r="I97">
+        <v>1.343029</v>
+      </c>
+      <c r="J97">
+        <v>32.946666669999999</v>
+      </c>
+      <c r="K97">
+        <v>160</v>
+      </c>
+      <c r="L97" t="s">
+        <v>30</v>
+      </c>
+      <c r="M97">
+        <v>4942</v>
+      </c>
+      <c r="N97" t="s">
+        <v>158</v>
+      </c>
+      <c r="O97">
+        <v>4017</v>
+      </c>
+      <c r="P97">
+        <v>1230.2713470000001</v>
+      </c>
+      <c r="Q97">
+        <v>150</v>
+      </c>
+      <c r="S97">
+        <v>32.946666999999998</v>
+      </c>
+      <c r="T97">
+        <v>3.7341299999999999</v>
+      </c>
+      <c r="U97">
+        <v>156</v>
+      </c>
+      <c r="V97">
+        <v>3.8834949999999999</v>
+      </c>
+      <c r="W97">
+        <v>31.679487000000002</v>
+      </c>
+      <c r="X97">
+        <v>104</v>
+      </c>
+      <c r="Y97">
+        <v>47.519230999999998</v>
+      </c>
+    </row>
+    <row r="98" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>25</v>
+      </c>
+      <c r="B98" t="s">
+        <v>26</v>
+      </c>
+      <c r="C98" t="s">
+        <v>161</v>
+      </c>
+      <c r="D98" t="s">
+        <v>38</v>
+      </c>
+      <c r="E98" t="s">
+        <v>29</v>
+      </c>
+      <c r="F98">
+        <v>112</v>
+      </c>
+      <c r="G98" t="s">
+        <v>42</v>
+      </c>
+      <c r="H98">
+        <v>2829</v>
+      </c>
+      <c r="I98">
+        <v>2.0901380000000001</v>
+      </c>
+      <c r="J98">
+        <v>43.705357139999997</v>
+      </c>
+      <c r="K98">
+        <v>160</v>
+      </c>
+      <c r="L98" t="s">
+        <v>30</v>
+      </c>
+      <c r="M98">
+        <v>4895</v>
+      </c>
+      <c r="N98" t="s">
+        <v>162</v>
+      </c>
+      <c r="O98">
+        <v>5913</v>
+      </c>
+      <c r="P98">
+        <v>827.83696899999995</v>
+      </c>
+      <c r="Q98">
+        <v>112</v>
+      </c>
+      <c r="S98">
+        <v>43.705356999999999</v>
+      </c>
+      <c r="T98">
+        <v>1.8941319999999999</v>
+      </c>
+      <c r="U98">
+        <v>146</v>
+      </c>
+      <c r="V98">
+        <v>2.4691360000000002</v>
+      </c>
+      <c r="W98">
+        <v>33.527397000000001</v>
+      </c>
+      <c r="X98">
+        <v>100</v>
+      </c>
+      <c r="Y98">
+        <v>48.95</v>
+      </c>
+    </row>
+    <row r="99" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>25</v>
+      </c>
+      <c r="B99" t="s">
+        <v>26</v>
+      </c>
+      <c r="C99" t="s">
+        <v>91</v>
+      </c>
+      <c r="D99" t="s">
+        <v>28</v>
+      </c>
+      <c r="E99" t="s">
+        <v>29</v>
+      </c>
+      <c r="F99">
+        <v>67</v>
+      </c>
+      <c r="G99" t="s">
+        <v>42</v>
+      </c>
+      <c r="H99">
+        <v>2389</v>
+      </c>
+      <c r="I99">
+        <v>1.3499369999999999</v>
+      </c>
+      <c r="J99">
+        <v>58.477611940000003</v>
+      </c>
+      <c r="K99">
+        <v>160</v>
+      </c>
+      <c r="L99" t="s">
+        <v>30</v>
+      </c>
+      <c r="M99">
+        <v>3918</v>
+      </c>
+      <c r="N99" t="s">
+        <v>92</v>
+      </c>
+      <c r="O99">
+        <v>3225</v>
+      </c>
+      <c r="P99">
+        <v>1214.8837209999999</v>
+      </c>
+      <c r="Q99">
+        <v>67</v>
+      </c>
+      <c r="S99">
+        <v>58.477612000000001</v>
+      </c>
+      <c r="T99">
+        <v>2.0775190000000001</v>
+      </c>
+      <c r="U99">
+        <v>75</v>
+      </c>
+      <c r="V99">
+        <v>2.3255810000000001</v>
+      </c>
+      <c r="W99">
+        <v>52.24</v>
+      </c>
+      <c r="X99">
+        <v>55</v>
+      </c>
+      <c r="Y99">
+        <v>71.236363999999995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>